<commit_message>
Add new Excel files and README updates for payroll analysis and dashboards
</commit_message>
<xml_diff>
--- a/Data_analysis_using_excel/Employee_Table.xlsx
+++ b/Data_analysis_using_excel/Employee_Table.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\VISHWAS SHARMA\Documents\Xcel_portfolio\Data_analysis_using_excel\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{E1DB532B-BD5B-43E0-A709-EB5A3073B11F}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{21B3050D-4567-43B2-A761-D1812C1A7BC9}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="10300" tabRatio="500" firstSheet="4" activeTab="7" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="11020" tabRatio="500" firstSheet="3" activeTab="6" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="employee" sheetId="1" r:id="rId1"/>
@@ -18,9 +18,8 @@
     <sheet name="subtotal" sheetId="2" r:id="rId3"/>
     <sheet name="Vlookup(2)" sheetId="4" r:id="rId4"/>
     <sheet name="vlookup(3)" sheetId="5" r:id="rId5"/>
-    <sheet name="approximate_match" sheetId="6" r:id="rId6"/>
-    <sheet name="hlookup(2)" sheetId="7" r:id="rId7"/>
-    <sheet name="Vlookup" sheetId="8" r:id="rId8"/>
+    <sheet name="hlookup(2)" sheetId="7" r:id="rId6"/>
+    <sheet name="Vlookup" sheetId="8" r:id="rId7"/>
   </sheets>
   <definedNames>
     <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">subtotal!$A$3:$H$15</definedName>
@@ -286,7 +285,7 @@
 </file>
 
 <file path=xl/metadata.xml><?xml version="1.0" encoding="utf-8"?>
-<metadata xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:xlrd="http://schemas.microsoft.com/office/spreadsheetml/2017/richdata" xmlns:xda="http://schemas.microsoft.com/office/spreadsheetml/2017/dynamicarray">
+<metadata xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:xda="http://schemas.microsoft.com/office/spreadsheetml/2017/dynamicarray">
   <metadataTypes count="1">
     <metadataType name="XLDAPR" minSupportedVersion="120000" copy="1" pasteAll="1" pasteValues="1" merge="1" splitFirst="1" rowColShift="1" clearFormats="1" clearComments="1" assign="1" coerce="1" cellMeta="1"/>
   </metadataTypes>
@@ -308,7 +307,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="496" uniqueCount="107">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="477" uniqueCount="90">
   <si>
     <t>Employee Table</t>
   </si>
@@ -533,57 +532,6 @@
   </si>
   <si>
     <t>Q: Find Age, Department and Mobile No. for an employee given Emp ID, using nested VLOOKUP with IFERROR.</t>
-  </si>
-  <si>
-    <t>Marks</t>
-  </si>
-  <si>
-    <t>Grade</t>
-  </si>
-  <si>
-    <t>Q: Find the Grade for a given Marks value using VLOOKUP with approximate match.</t>
-  </si>
-  <si>
-    <t>F</t>
-  </si>
-  <si>
-    <t>Given Marks:</t>
-  </si>
-  <si>
-    <t>D</t>
-  </si>
-  <si>
-    <t>C</t>
-  </si>
-  <si>
-    <t>B</t>
-  </si>
-  <si>
-    <t>A</t>
-  </si>
-  <si>
-    <t>Q: Find the sales figure for a given Product and Month using VLOOKUP + MATCH.</t>
-  </si>
-  <si>
-    <t>Mango</t>
-  </si>
-  <si>
-    <t>Jan</t>
-  </si>
-  <si>
-    <t>Product</t>
-  </si>
-  <si>
-    <t>Feb</t>
-  </si>
-  <si>
-    <t>Mar</t>
-  </si>
-  <si>
-    <t>Apple</t>
-  </si>
-  <si>
-    <t>Banana</t>
   </si>
   <si>
     <t>Given Emp ID:</t>
@@ -1387,7 +1335,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="140">
+  <cellXfs count="135">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="3" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
@@ -1426,9 +1374,6 @@
     </xf>
     <xf numFmtId="1" fontId="10" fillId="0" borderId="3" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="2" fillId="3" borderId="12" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="12" xfId="0" applyFont="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="12" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
@@ -1506,14 +1451,6 @@
       <alignment vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="7" borderId="26" xfId="0" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="0" fillId="7" borderId="28" xfId="0" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="8" fillId="7" borderId="28" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="right"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="7" borderId="30" xfId="0" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="4" fillId="6" borderId="23" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
     <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment vertical="center"/>
     </xf>
@@ -1622,6 +1559,9 @@
     <xf numFmtId="0" fontId="10" fillId="6" borderId="24" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="10" fillId="0" borderId="24" xfId="0" applyFont="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="10" fillId="0" borderId="25" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="9" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
     <xf numFmtId="0" fontId="4" fillId="6" borderId="23" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
@@ -1660,9 +1600,6 @@
     </xf>
     <xf numFmtId="0" fontId="9" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="9" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -1949,36 +1886,36 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:25" ht="14.25" customHeight="1">
-      <c r="A1" s="130" t="s">
+      <c r="A1" s="126" t="s">
         <v>0</v>
       </c>
-      <c r="B1" s="130"/>
-      <c r="C1" s="130"/>
-      <c r="D1" s="130"/>
-      <c r="E1" s="130"/>
-      <c r="F1" s="130"/>
-      <c r="G1" s="130"/>
-      <c r="H1" s="130"/>
+      <c r="B1" s="126"/>
+      <c r="C1" s="126"/>
+      <c r="D1" s="126"/>
+      <c r="E1" s="126"/>
+      <c r="F1" s="126"/>
+      <c r="G1" s="126"/>
+      <c r="H1" s="126"/>
     </row>
     <row r="2" spans="1:25" ht="14.25" customHeight="1" thickBot="1">
-      <c r="A2" s="130"/>
-      <c r="B2" s="130"/>
-      <c r="C2" s="130"/>
-      <c r="D2" s="130"/>
-      <c r="E2" s="130"/>
-      <c r="F2" s="130"/>
-      <c r="G2" s="130"/>
-      <c r="H2" s="130"/>
+      <c r="A2" s="126"/>
+      <c r="B2" s="126"/>
+      <c r="C2" s="126"/>
+      <c r="D2" s="126"/>
+      <c r="E2" s="126"/>
+      <c r="F2" s="126"/>
+      <c r="G2" s="126"/>
+      <c r="H2" s="126"/>
       <c r="U2" s="1" t="s">
         <v>35</v>
       </c>
       <c r="V2" s="1" t="s">
         <v>36</v>
       </c>
-      <c r="W2" s="129" t="s">
+      <c r="W2" s="125" t="s">
         <v>37</v>
       </c>
-      <c r="X2" s="129"/>
+      <c r="X2" s="125"/>
       <c r="Y2" s="1" t="s">
         <v>38</v>
       </c>
@@ -2008,19 +1945,19 @@
       <c r="H3" s="1" t="s">
         <v>8</v>
       </c>
-      <c r="K3" s="131" t="s">
+      <c r="K3" s="127" t="s">
         <v>30</v>
       </c>
-      <c r="L3" s="132"/>
-      <c r="M3" s="132"/>
-      <c r="N3" s="132"/>
-      <c r="O3" s="132"/>
-      <c r="P3" s="132"/>
-      <c r="Q3" s="133"/>
+      <c r="L3" s="128"/>
+      <c r="M3" s="128"/>
+      <c r="N3" s="128"/>
+      <c r="O3" s="128"/>
+      <c r="P3" s="128"/>
+      <c r="Q3" s="129"/>
       <c r="U3" s="6">
         <v>1</v>
       </c>
-      <c r="V3" s="120" t="s">
+      <c r="V3" s="115" t="s">
         <v>39</v>
       </c>
       <c r="W3" s="6"/>
@@ -2055,38 +1992,38 @@
       <c r="H4" s="5">
         <v>8877456987</v>
       </c>
-      <c r="K4" s="110" t="str" cm="1">
+      <c r="K4" s="105" t="str" cm="1">
         <f t="array" ref="K4:Q4">_xlfn.XLOOKUP(A4,A3:A15,B3:H15)</f>
         <v>Kapil Sharma</v>
       </c>
-      <c r="L4" s="111">
+      <c r="L4" s="106">
         <v>26</v>
       </c>
-      <c r="M4" s="111" t="str">
+      <c r="M4" s="106" t="str">
         <v>Engineer</v>
       </c>
-      <c r="N4" s="111" t="str">
+      <c r="N4" s="106" t="str">
         <v>Technical</v>
       </c>
-      <c r="O4" s="111">
+      <c r="O4" s="106">
         <v>26500</v>
       </c>
-      <c r="P4" s="111" t="str">
+      <c r="P4" s="106" t="str">
         <v>Indore</v>
       </c>
-      <c r="Q4" s="117">
+      <c r="Q4" s="112">
         <v>8877456987</v>
       </c>
       <c r="U4" s="6">
         <v>2</v>
       </c>
-      <c r="V4" s="120" t="s">
+      <c r="V4" s="115" t="s">
         <v>40</v>
       </c>
-      <c r="W4" s="121">
+      <c r="W4" s="116">
         <v>20012</v>
       </c>
-      <c r="X4" s="121" t="s">
+      <c r="X4" s="116" t="s">
         <v>3</v>
       </c>
       <c r="Y4" s="6">
@@ -2122,7 +2059,7 @@
       <c r="U5" s="6">
         <v>3</v>
       </c>
-      <c r="V5" s="120" t="s">
+      <c r="V5" s="115" t="s">
         <v>41</v>
       </c>
       <c r="W5" s="6"/>
@@ -2160,7 +2097,7 @@
       <c r="U6" s="6">
         <v>4</v>
       </c>
-      <c r="V6" s="120" t="s">
+      <c r="V6" s="115" t="s">
         <v>42</v>
       </c>
       <c r="W6" s="6"/>
@@ -2198,7 +2135,7 @@
       <c r="U7" s="6">
         <v>5</v>
       </c>
-      <c r="V7" s="120" t="s">
+      <c r="V7" s="115" t="s">
         <v>43</v>
       </c>
       <c r="W7" s="6"/>
@@ -2221,10 +2158,10 @@
       <c r="D8" s="3" t="s">
         <v>10</v>
       </c>
-      <c r="E8" s="21" t="s">
+      <c r="E8" s="20" t="s">
         <v>11</v>
       </c>
-      <c r="F8" s="118">
+      <c r="F8" s="113">
         <v>20000</v>
       </c>
       <c r="G8" s="19" t="s">
@@ -2236,7 +2173,7 @@
       <c r="U8" s="6">
         <v>6</v>
       </c>
-      <c r="V8" s="120" t="s">
+      <c r="V8" s="115" t="s">
         <v>44</v>
       </c>
       <c r="W8" s="6"/>
@@ -2274,7 +2211,7 @@
       <c r="U9" s="6">
         <v>7</v>
       </c>
-      <c r="V9" s="120" t="s">
+      <c r="V9" s="115" t="s">
         <v>45</v>
       </c>
       <c r="W9" s="6"/>
@@ -2312,7 +2249,7 @@
       <c r="U10" s="6">
         <v>8</v>
       </c>
-      <c r="V10" s="120" t="s">
+      <c r="V10" s="115" t="s">
         <v>46</v>
       </c>
       <c r="W10" s="6"/>
@@ -2347,19 +2284,19 @@
       <c r="H11" s="5">
         <v>8745968745</v>
       </c>
-      <c r="K11" s="113" t="s">
+      <c r="K11" s="108" t="s">
         <v>25</v>
       </c>
-      <c r="L11" s="114"/>
-      <c r="M11" s="114"/>
-      <c r="N11" s="114"/>
-      <c r="O11" s="114"/>
-      <c r="P11" s="114"/>
-      <c r="Q11" s="25"/>
+      <c r="L11" s="109"/>
+      <c r="M11" s="109"/>
+      <c r="N11" s="109"/>
+      <c r="O11" s="109"/>
+      <c r="P11" s="109"/>
+      <c r="Q11" s="24"/>
       <c r="U11" s="6">
         <v>9</v>
       </c>
-      <c r="V11" s="120" t="s">
+      <c r="V11" s="115" t="s">
         <v>47</v>
       </c>
       <c r="W11" s="6"/>
@@ -2394,23 +2331,23 @@
       <c r="H12" s="5">
         <v>9874569874</v>
       </c>
-      <c r="K12" s="56"/>
-      <c r="L12" s="122" t="str">
+      <c r="K12" s="55"/>
+      <c r="L12" s="117" t="str">
         <f t="array" ref="L12:N24">CHOOSE({1,2,3},F3:F15,C3:C15,A3:A15)</f>
         <v>Salary</v>
       </c>
-      <c r="M12" s="123" t="str">
+      <c r="M12" s="118" t="str">
         <v>Age</v>
       </c>
-      <c r="N12" s="123" t="str">
+      <c r="N12" s="118" t="str">
         <v>Emp. ID</v>
       </c>
-      <c r="O12" s="124"/>
-      <c r="P12" s="125"/>
+      <c r="O12" s="119"/>
+      <c r="P12" s="120"/>
       <c r="U12" s="6">
         <v>10</v>
       </c>
-      <c r="V12" s="120" t="s">
+      <c r="V12" s="115" t="s">
         <v>48</v>
       </c>
       <c r="W12" s="6"/>
@@ -2445,22 +2382,22 @@
       <c r="H13" s="5">
         <v>8574965874</v>
       </c>
-      <c r="K13" s="56"/>
-      <c r="L13" s="107">
+      <c r="K13" s="55"/>
+      <c r="L13" s="102">
         <v>26500</v>
       </c>
-      <c r="M13" s="108">
+      <c r="M13" s="103">
         <v>26</v>
       </c>
-      <c r="N13" s="108">
+      <c r="N13" s="103">
         <v>20012</v>
       </c>
-      <c r="O13" s="108"/>
-      <c r="P13" s="109"/>
+      <c r="O13" s="103"/>
+      <c r="P13" s="104"/>
       <c r="U13" s="6">
         <v>11</v>
       </c>
-      <c r="V13" s="120" t="s">
+      <c r="V13" s="115" t="s">
         <v>49</v>
       </c>
       <c r="W13" s="6"/>
@@ -2495,22 +2432,22 @@
       <c r="H14" s="5">
         <v>8521479632</v>
       </c>
-      <c r="K14" s="56"/>
-      <c r="L14" s="107">
+      <c r="K14" s="55"/>
+      <c r="L14" s="102">
         <v>13000</v>
       </c>
-      <c r="M14" s="108">
+      <c r="M14" s="103">
         <v>25</v>
       </c>
-      <c r="N14" s="108">
+      <c r="N14" s="103">
         <v>20013</v>
       </c>
-      <c r="O14" s="108"/>
-      <c r="P14" s="109"/>
+      <c r="O14" s="103"/>
+      <c r="P14" s="104"/>
       <c r="U14" s="6">
         <v>12</v>
       </c>
-      <c r="V14" s="120" t="s">
+      <c r="V14" s="115" t="s">
         <v>50</v>
       </c>
       <c r="W14" s="6"/>
@@ -2545,25 +2482,25 @@
       <c r="H15" s="5">
         <v>8569745623</v>
       </c>
-      <c r="K15" s="56"/>
-      <c r="L15" s="107">
+      <c r="K15" s="55"/>
+      <c r="L15" s="102">
         <v>20000</v>
       </c>
-      <c r="M15" s="108">
+      <c r="M15" s="103">
         <v>28</v>
       </c>
-      <c r="N15" s="108">
+      <c r="N15" s="103">
         <v>20014</v>
       </c>
-      <c r="O15" s="108"/>
-      <c r="P15" s="109"/>
+      <c r="O15" s="103"/>
+      <c r="P15" s="104"/>
       <c r="U15" s="6">
         <v>13</v>
       </c>
-      <c r="V15" s="120" t="s">
+      <c r="V15" s="115" t="s">
         <v>51</v>
       </c>
-      <c r="W15" s="121">
+      <c r="W15" s="116">
         <v>40500</v>
       </c>
       <c r="X15" s="6"/>
@@ -2573,22 +2510,22 @@
       </c>
     </row>
     <row r="16" spans="1:25" ht="14.25" customHeight="1">
-      <c r="K16" s="56"/>
-      <c r="L16" s="107">
+      <c r="K16" s="55"/>
+      <c r="L16" s="102">
         <v>15000</v>
       </c>
-      <c r="M16" s="108">
+      <c r="M16" s="103">
         <v>27</v>
       </c>
-      <c r="N16" s="108">
+      <c r="N16" s="103">
         <v>20015</v>
       </c>
-      <c r="O16" s="108"/>
-      <c r="P16" s="109"/>
+      <c r="O16" s="103"/>
+      <c r="P16" s="104"/>
       <c r="U16" s="6">
         <v>14</v>
       </c>
-      <c r="V16" s="120" t="s">
+      <c r="V16" s="115" t="s">
         <v>52</v>
       </c>
       <c r="W16" s="6"/>
@@ -2599,22 +2536,22 @@
       </c>
     </row>
     <row r="17" spans="2:25" ht="14.25" customHeight="1">
-      <c r="K17" s="56"/>
-      <c r="L17" s="107">
+      <c r="K17" s="55"/>
+      <c r="L17" s="102">
         <v>20000</v>
       </c>
-      <c r="M17" s="108">
+      <c r="M17" s="103">
         <v>25</v>
       </c>
-      <c r="N17" s="108">
+      <c r="N17" s="103">
         <v>20016</v>
       </c>
-      <c r="O17" s="108"/>
-      <c r="P17" s="109"/>
+      <c r="O17" s="103"/>
+      <c r="P17" s="104"/>
       <c r="U17" s="6">
         <v>15</v>
       </c>
-      <c r="V17" s="120" t="s">
+      <c r="V17" s="115" t="s">
         <v>53</v>
       </c>
       <c r="W17" s="6"/>
@@ -2625,115 +2562,115 @@
       </c>
     </row>
     <row r="18" spans="2:25" ht="14.25" customHeight="1">
-      <c r="K18" s="56"/>
-      <c r="L18" s="107">
+      <c r="K18" s="55"/>
+      <c r="L18" s="102">
         <v>33000</v>
       </c>
-      <c r="M18" s="108">
+      <c r="M18" s="103">
         <v>26</v>
       </c>
-      <c r="N18" s="108">
+      <c r="N18" s="103">
         <v>20017</v>
       </c>
-      <c r="O18" s="108"/>
-      <c r="P18" s="109"/>
+      <c r="O18" s="103"/>
+      <c r="P18" s="104"/>
     </row>
     <row r="19" spans="2:25" ht="14.25" customHeight="1">
-      <c r="K19" s="56"/>
-      <c r="L19" s="107">
+      <c r="K19" s="55"/>
+      <c r="L19" s="102">
         <v>21000</v>
       </c>
-      <c r="M19" s="108">
+      <c r="M19" s="103">
         <v>25</v>
       </c>
-      <c r="N19" s="108">
+      <c r="N19" s="103">
         <v>20018</v>
       </c>
-      <c r="O19" s="108"/>
-      <c r="P19" s="109"/>
+      <c r="O19" s="103"/>
+      <c r="P19" s="104"/>
     </row>
     <row r="20" spans="2:25" ht="14.25" customHeight="1">
-      <c r="K20" s="56"/>
-      <c r="L20" s="107">
+      <c r="K20" s="55"/>
+      <c r="L20" s="102">
         <v>31500</v>
       </c>
-      <c r="M20" s="108">
+      <c r="M20" s="103">
         <v>26</v>
       </c>
-      <c r="N20" s="108">
+      <c r="N20" s="103">
         <v>20019</v>
       </c>
-      <c r="O20" s="108"/>
-      <c r="P20" s="109"/>
+      <c r="O20" s="103"/>
+      <c r="P20" s="104"/>
     </row>
     <row r="21" spans="2:25" ht="21" customHeight="1">
-      <c r="K21" s="56"/>
-      <c r="L21" s="107">
+      <c r="K21" s="55"/>
+      <c r="L21" s="102">
         <v>40500</v>
       </c>
-      <c r="M21" s="108">
+      <c r="M21" s="103">
         <v>28</v>
       </c>
-      <c r="N21" s="108">
+      <c r="N21" s="103">
         <v>20020</v>
       </c>
-      <c r="O21" s="108"/>
-      <c r="P21" s="109"/>
+      <c r="O21" s="103"/>
+      <c r="P21" s="104"/>
     </row>
     <row r="22" spans="2:25" ht="14.25" customHeight="1">
-      <c r="K22" s="56"/>
-      <c r="L22" s="107">
+      <c r="K22" s="55"/>
+      <c r="L22" s="102">
         <v>25500</v>
       </c>
-      <c r="M22" s="108">
+      <c r="M22" s="103">
         <v>27</v>
       </c>
-      <c r="N22" s="108">
+      <c r="N22" s="103">
         <v>20021</v>
       </c>
-      <c r="O22" s="108"/>
-      <c r="P22" s="109"/>
+      <c r="O22" s="103"/>
+      <c r="P22" s="104"/>
     </row>
     <row r="23" spans="2:25" ht="14.25" customHeight="1" thickBot="1">
-      <c r="K23" s="56"/>
-      <c r="L23" s="107">
+      <c r="K23" s="55"/>
+      <c r="L23" s="102">
         <v>18000</v>
       </c>
-      <c r="M23" s="108">
+      <c r="M23" s="103">
         <v>26</v>
       </c>
-      <c r="N23" s="108">
+      <c r="N23" s="103">
         <v>20022</v>
       </c>
-      <c r="O23" s="108"/>
-      <c r="P23" s="109"/>
+      <c r="O23" s="103"/>
+      <c r="P23" s="104"/>
     </row>
     <row r="24" spans="2:25" ht="21" customHeight="1" thickBot="1">
-      <c r="B24" s="126" t="s">
+      <c r="B24" s="122" t="s">
         <v>31</v>
       </c>
-      <c r="C24" s="127"/>
-      <c r="D24" s="127"/>
-      <c r="E24" s="127"/>
-      <c r="F24" s="127"/>
-      <c r="G24" s="127"/>
-      <c r="H24" s="127"/>
-      <c r="I24" s="128"/>
-      <c r="K24" s="57"/>
-      <c r="L24" s="110">
+      <c r="C24" s="123"/>
+      <c r="D24" s="123"/>
+      <c r="E24" s="123"/>
+      <c r="F24" s="123"/>
+      <c r="G24" s="123"/>
+      <c r="H24" s="123"/>
+      <c r="I24" s="124"/>
+      <c r="K24" s="56"/>
+      <c r="L24" s="105">
         <v>21000</v>
       </c>
-      <c r="M24" s="111">
+      <c r="M24" s="106">
         <v>27</v>
       </c>
-      <c r="N24" s="111">
+      <c r="N24" s="106">
         <v>20023</v>
       </c>
-      <c r="O24" s="111"/>
-      <c r="P24" s="112"/>
+      <c r="O24" s="106"/>
+      <c r="P24" s="107"/>
     </row>
     <row r="25" spans="2:25" ht="14.25" customHeight="1">
-      <c r="B25" s="56" t="str">
+      <c r="B25" s="55" t="str">
         <f t="array" ref="B25:I34">_xlfn._xlws.FILTER(A3:H15,C3:C15&gt;25)</f>
         <v>Emp. ID</v>
       </c>
@@ -2755,12 +2692,12 @@
       <c r="H25" t="str">
         <v>Place</v>
       </c>
-      <c r="I25" s="55" t="str">
+      <c r="I25" s="54" t="str">
         <v>Mob.No.</v>
       </c>
     </row>
     <row r="26" spans="2:25" ht="14.25" customHeight="1">
-      <c r="B26" s="56">
+      <c r="B26" s="55">
         <v>20012</v>
       </c>
       <c r="C26" t="str">
@@ -2781,12 +2718,12 @@
       <c r="H26" t="str">
         <v>Indore</v>
       </c>
-      <c r="I26" s="119">
+      <c r="I26" s="114">
         <v>8877456987</v>
       </c>
     </row>
     <row r="27" spans="2:25" ht="14.25" customHeight="1">
-      <c r="B27" s="56">
+      <c r="B27" s="55">
         <v>20014</v>
       </c>
       <c r="C27" t="str">
@@ -2807,12 +2744,12 @@
       <c r="H27" t="str">
         <v>Indore</v>
       </c>
-      <c r="I27" s="119">
+      <c r="I27" s="114">
         <v>7584963214</v>
       </c>
     </row>
     <row r="28" spans="2:25" ht="14.25" customHeight="1">
-      <c r="B28" s="56">
+      <c r="B28" s="55">
         <v>20015</v>
       </c>
       <c r="C28" t="str">
@@ -2833,12 +2770,12 @@
       <c r="H28" t="str">
         <v>Bhopal</v>
       </c>
-      <c r="I28" s="119">
+      <c r="I28" s="114">
         <v>7788994455</v>
       </c>
     </row>
     <row r="29" spans="2:25" ht="14.25" customHeight="1">
-      <c r="B29" s="56">
+      <c r="B29" s="55">
         <v>20017</v>
       </c>
       <c r="C29" t="str">
@@ -2859,12 +2796,12 @@
       <c r="H29" t="str">
         <v>Bhopal</v>
       </c>
-      <c r="I29" s="119">
+      <c r="I29" s="114">
         <v>9874563214</v>
       </c>
     </row>
     <row r="30" spans="2:25" ht="14.25" customHeight="1">
-      <c r="B30" s="56">
+      <c r="B30" s="55">
         <v>20019</v>
       </c>
       <c r="C30" t="str">
@@ -2885,12 +2822,12 @@
       <c r="H30" t="str">
         <v>Bhopal</v>
       </c>
-      <c r="I30" s="119">
+      <c r="I30" s="114">
         <v>8745968745</v>
       </c>
     </row>
     <row r="31" spans="2:25" ht="14.25" customHeight="1">
-      <c r="B31" s="56">
+      <c r="B31" s="55">
         <v>20020</v>
       </c>
       <c r="C31" t="str">
@@ -2911,12 +2848,12 @@
       <c r="H31" t="str">
         <v>Indore</v>
       </c>
-      <c r="I31" s="119">
+      <c r="I31" s="114">
         <v>9874569874</v>
       </c>
     </row>
     <row r="32" spans="2:25" ht="14.25" customHeight="1">
-      <c r="B32" s="56">
+      <c r="B32" s="55">
         <v>20021</v>
       </c>
       <c r="C32" t="str">
@@ -2937,12 +2874,12 @@
       <c r="H32" t="str">
         <v>ujjain</v>
       </c>
-      <c r="I32" s="119">
+      <c r="I32" s="114">
         <v>8574965874</v>
       </c>
     </row>
     <row r="33" spans="2:9" ht="14.25" customHeight="1">
-      <c r="B33" s="56">
+      <c r="B33" s="55">
         <v>20022</v>
       </c>
       <c r="C33" t="str">
@@ -2963,50 +2900,50 @@
       <c r="H33" t="str">
         <v>ujjain</v>
       </c>
-      <c r="I33" s="119">
+      <c r="I33" s="114">
         <v>8521479632</v>
       </c>
     </row>
     <row r="34" spans="2:9" ht="14.25" customHeight="1" thickBot="1">
-      <c r="B34" s="57">
+      <c r="B34" s="56">
         <v>20023</v>
       </c>
-      <c r="C34" s="58" t="str">
+      <c r="C34" s="57" t="str">
         <v>Janwi Rai</v>
       </c>
-      <c r="D34" s="58">
+      <c r="D34" s="57">
         <v>27</v>
       </c>
-      <c r="E34" s="58" t="str">
+      <c r="E34" s="57" t="str">
         <v>CAD Designer</v>
       </c>
-      <c r="F34" s="58" t="str">
+      <c r="F34" s="57" t="str">
         <v>Technical</v>
       </c>
-      <c r="G34" s="58">
+      <c r="G34" s="57">
         <v>21000</v>
       </c>
-      <c r="H34" s="58" t="str">
+      <c r="H34" s="57" t="str">
         <v>Indore</v>
       </c>
-      <c r="I34" s="59">
+      <c r="I34" s="58">
         <v>8569745623</v>
       </c>
     </row>
     <row r="35" spans="2:9" ht="21" customHeight="1">
-      <c r="B35" s="126" t="s">
+      <c r="B35" s="122" t="s">
         <v>32</v>
       </c>
-      <c r="C35" s="127"/>
-      <c r="D35" s="127"/>
-      <c r="E35" s="127"/>
-      <c r="F35" s="127"/>
-      <c r="G35" s="127"/>
-      <c r="H35" s="127"/>
-      <c r="I35" s="128"/>
+      <c r="C35" s="123"/>
+      <c r="D35" s="123"/>
+      <c r="E35" s="123"/>
+      <c r="F35" s="123"/>
+      <c r="G35" s="123"/>
+      <c r="H35" s="123"/>
+      <c r="I35" s="124"/>
     </row>
     <row r="36" spans="2:9" ht="14.25" customHeight="1">
-      <c r="B36" s="56">
+      <c r="B36" s="55">
         <f t="array" ref="B36:I42">_xlfn._xlws.FILTER(A3:H15,E3:E15="Technical")</f>
         <v>20012</v>
       </c>
@@ -3028,12 +2965,12 @@
       <c r="H36" t="str">
         <v>Indore</v>
       </c>
-      <c r="I36" s="119">
+      <c r="I36" s="114">
         <v>8877456987</v>
       </c>
     </row>
     <row r="37" spans="2:9" ht="14.25" customHeight="1">
-      <c r="B37" s="56">
+      <c r="B37" s="55">
         <v>20014</v>
       </c>
       <c r="C37" t="str">
@@ -3054,12 +2991,12 @@
       <c r="H37" t="str">
         <v>Indore</v>
       </c>
-      <c r="I37" s="119">
+      <c r="I37" s="114">
         <v>7584963214</v>
       </c>
     </row>
     <row r="38" spans="2:9" ht="14.25" customHeight="1">
-      <c r="B38" s="56">
+      <c r="B38" s="55">
         <v>20016</v>
       </c>
       <c r="C38" t="str">
@@ -3080,12 +3017,12 @@
       <c r="H38" t="str">
         <v>ujjain</v>
       </c>
-      <c r="I38" s="119">
+      <c r="I38" s="114">
         <v>8798654512</v>
       </c>
     </row>
     <row r="39" spans="2:9" ht="14.25" customHeight="1">
-      <c r="B39" s="56">
+      <c r="B39" s="55">
         <v>20017</v>
       </c>
       <c r="C39" t="str">
@@ -3106,12 +3043,12 @@
       <c r="H39" t="str">
         <v>Bhopal</v>
       </c>
-      <c r="I39" s="119">
+      <c r="I39" s="114">
         <v>9874563214</v>
       </c>
     </row>
     <row r="40" spans="2:9" ht="14.25" customHeight="1">
-      <c r="B40" s="56">
+      <c r="B40" s="55">
         <v>20018</v>
       </c>
       <c r="C40" t="str">
@@ -3132,12 +3069,12 @@
       <c r="H40" t="str">
         <v>Indore</v>
       </c>
-      <c r="I40" s="119">
+      <c r="I40" s="114">
         <v>8974563214</v>
       </c>
     </row>
     <row r="41" spans="2:9" ht="14.25" customHeight="1">
-      <c r="B41" s="56">
+      <c r="B41" s="55">
         <v>20021</v>
       </c>
       <c r="C41" t="str">
@@ -3158,50 +3095,50 @@
       <c r="H41" t="str">
         <v>ujjain</v>
       </c>
-      <c r="I41" s="119">
+      <c r="I41" s="114">
         <v>8574965874</v>
       </c>
     </row>
     <row r="42" spans="2:9" ht="14.25" customHeight="1" thickBot="1">
-      <c r="B42" s="57">
+      <c r="B42" s="56">
         <v>20023</v>
       </c>
-      <c r="C42" s="58" t="str">
+      <c r="C42" s="57" t="str">
         <v>Janwi Rai</v>
       </c>
-      <c r="D42" s="58">
+      <c r="D42" s="57">
         <v>27</v>
       </c>
-      <c r="E42" s="58" t="str">
+      <c r="E42" s="57" t="str">
         <v>CAD Designer</v>
       </c>
-      <c r="F42" s="58" t="str">
+      <c r="F42" s="57" t="str">
         <v>Technical</v>
       </c>
-      <c r="G42" s="58">
+      <c r="G42" s="57">
         <v>21000</v>
       </c>
-      <c r="H42" s="58" t="str">
+      <c r="H42" s="57" t="str">
         <v>Indore</v>
       </c>
-      <c r="I42" s="59">
+      <c r="I42" s="58">
         <v>8569745623</v>
       </c>
     </row>
     <row r="43" spans="2:9" ht="21" customHeight="1">
-      <c r="B43" s="126" t="s">
+      <c r="B43" s="122" t="s">
         <v>33</v>
       </c>
-      <c r="C43" s="127"/>
-      <c r="D43" s="127"/>
-      <c r="E43" s="127"/>
-      <c r="F43" s="127"/>
-      <c r="G43" s="127"/>
-      <c r="H43" s="127"/>
-      <c r="I43" s="128"/>
+      <c r="C43" s="123"/>
+      <c r="D43" s="123"/>
+      <c r="E43" s="123"/>
+      <c r="F43" s="123"/>
+      <c r="G43" s="123"/>
+      <c r="H43" s="123"/>
+      <c r="I43" s="124"/>
     </row>
     <row r="44" spans="2:9" ht="14.25" customHeight="1">
-      <c r="B44" s="56">
+      <c r="B44" s="55">
         <f t="array" ref="B44:I47">_xlfn._xlws.FILTER(A3:H15,G3:G15="Bhopal")</f>
         <v>20013</v>
       </c>
@@ -3223,12 +3160,12 @@
       <c r="H44" t="str">
         <v>Bhopal</v>
       </c>
-      <c r="I44" s="119">
+      <c r="I44" s="114">
         <v>8569741235</v>
       </c>
     </row>
     <row r="45" spans="2:9" ht="14.25" customHeight="1">
-      <c r="B45" s="56">
+      <c r="B45" s="55">
         <v>20015</v>
       </c>
       <c r="C45" t="str">
@@ -3249,12 +3186,12 @@
       <c r="H45" t="str">
         <v>Bhopal</v>
       </c>
-      <c r="I45" s="119">
+      <c r="I45" s="114">
         <v>7788994455</v>
       </c>
     </row>
     <row r="46" spans="2:9" ht="14.25" customHeight="1">
-      <c r="B46" s="56">
+      <c r="B46" s="55">
         <v>20017</v>
       </c>
       <c r="C46" t="str">
@@ -3275,50 +3212,50 @@
       <c r="H46" t="str">
         <v>Bhopal</v>
       </c>
-      <c r="I46" s="119">
+      <c r="I46" s="114">
         <v>9874563214</v>
       </c>
     </row>
     <row r="47" spans="2:9" ht="14.25" customHeight="1" thickBot="1">
-      <c r="B47" s="57">
+      <c r="B47" s="56">
         <v>20019</v>
       </c>
-      <c r="C47" s="58" t="str">
+      <c r="C47" s="57" t="str">
         <v>Deepak Singh</v>
       </c>
-      <c r="D47" s="58">
+      <c r="D47" s="57">
         <v>26</v>
       </c>
-      <c r="E47" s="58" t="str">
+      <c r="E47" s="57" t="str">
         <v>Accountant</v>
       </c>
-      <c r="F47" s="58" t="str">
+      <c r="F47" s="57" t="str">
         <v>Finance</v>
       </c>
-      <c r="G47" s="58">
+      <c r="G47" s="57">
         <v>31500</v>
       </c>
-      <c r="H47" s="58" t="str">
+      <c r="H47" s="57" t="str">
         <v>Bhopal</v>
       </c>
-      <c r="I47" s="59">
+      <c r="I47" s="58">
         <v>8745968745</v>
       </c>
     </row>
     <row r="48" spans="2:9" ht="21" customHeight="1">
-      <c r="B48" s="126" t="s">
+      <c r="B48" s="122" t="s">
         <v>34</v>
       </c>
-      <c r="C48" s="127"/>
-      <c r="D48" s="127"/>
-      <c r="E48" s="127"/>
-      <c r="F48" s="127"/>
-      <c r="G48" s="127"/>
-      <c r="H48" s="127"/>
-      <c r="I48" s="128"/>
+      <c r="C48" s="123"/>
+      <c r="D48" s="123"/>
+      <c r="E48" s="123"/>
+      <c r="F48" s="123"/>
+      <c r="G48" s="123"/>
+      <c r="H48" s="123"/>
+      <c r="I48" s="124"/>
     </row>
     <row r="49" spans="2:9" ht="14.25" customHeight="1">
-      <c r="B49" s="56" t="str">
+      <c r="B49" s="55" t="str">
         <f t="array" ref="B49:I52">_xlfn._xlws.FILTER(A3:H15,F3:F15&gt;30000)</f>
         <v>Emp. ID</v>
       </c>
@@ -3340,12 +3277,12 @@
       <c r="H49" t="str">
         <v>Place</v>
       </c>
-      <c r="I49" s="55" t="str">
+      <c r="I49" s="54" t="str">
         <v>Mob.No.</v>
       </c>
     </row>
     <row r="50" spans="2:9" ht="14.25" customHeight="1">
-      <c r="B50" s="56">
+      <c r="B50" s="55">
         <v>20017</v>
       </c>
       <c r="C50" t="str">
@@ -3366,12 +3303,12 @@
       <c r="H50" t="str">
         <v>Bhopal</v>
       </c>
-      <c r="I50" s="119">
+      <c r="I50" s="114">
         <v>9874563214</v>
       </c>
     </row>
     <row r="51" spans="2:9" ht="14.25" customHeight="1">
-      <c r="B51" s="56">
+      <c r="B51" s="55">
         <v>20019</v>
       </c>
       <c r="C51" t="str">
@@ -3392,33 +3329,33 @@
       <c r="H51" t="str">
         <v>Bhopal</v>
       </c>
-      <c r="I51" s="119">
+      <c r="I51" s="114">
         <v>8745968745</v>
       </c>
     </row>
     <row r="52" spans="2:9" ht="14.25" customHeight="1" thickBot="1">
-      <c r="B52" s="57">
+      <c r="B52" s="56">
         <v>20020</v>
       </c>
-      <c r="C52" s="58" t="str">
+      <c r="C52" s="57" t="str">
         <v>Vikas Patel</v>
       </c>
-      <c r="D52" s="58">
+      <c r="D52" s="57">
         <v>28</v>
       </c>
-      <c r="E52" s="58" t="str">
+      <c r="E52" s="57" t="str">
         <v>Accountant</v>
       </c>
-      <c r="F52" s="58" t="str">
+      <c r="F52" s="57" t="str">
         <v>Finance</v>
       </c>
-      <c r="G52" s="58">
+      <c r="G52" s="57">
         <v>40500</v>
       </c>
-      <c r="H52" s="58" t="str">
+      <c r="H52" s="57" t="str">
         <v>Indore</v>
       </c>
-      <c r="I52" s="59">
+      <c r="I52" s="58">
         <v>9874569874</v>
       </c>
     </row>
@@ -3476,89 +3413,89 @@
   </cols>
   <sheetData>
     <row r="1" spans="2:10" ht="41.25" customHeight="1">
-      <c r="B1" s="64" t="s">
-        <v>103</v>
-      </c>
-      <c r="C1" s="54">
+      <c r="B1" s="63" t="s">
+        <v>86</v>
+      </c>
+      <c r="C1" s="53">
         <f>VLOOKUP(B2,employee!A3:H15,6,0)</f>
         <v>20000</v>
       </c>
       <c r="D1" s="12"/>
     </row>
     <row r="2" spans="2:10" ht="14.25" customHeight="1" thickBot="1">
-      <c r="B2" s="65">
+      <c r="B2" s="64">
         <v>20016</v>
       </c>
-      <c r="C2" s="105"/>
+      <c r="C2" s="100"/>
     </row>
     <row r="3" spans="2:10" ht="27.75" customHeight="1">
-      <c r="B3" s="64" t="s">
-        <v>104</v>
-      </c>
-      <c r="C3" s="79" t="str">
+      <c r="B3" s="63" t="s">
+        <v>87</v>
+      </c>
+      <c r="C3" s="74" t="str">
         <f t="array" ref="C3:I3">VLOOKUP(B4,Vlookup!A3:H15,{2,3,4,5,6,7,8},0)</f>
         <v>Sunil Grover</v>
       </c>
-      <c r="D3" s="79">
+      <c r="D3" s="74">
         <v>25</v>
       </c>
-      <c r="E3" s="79" t="str">
+      <c r="E3" s="74" t="str">
         <v>Accountant</v>
       </c>
-      <c r="F3" s="79" t="str">
+      <c r="F3" s="74" t="str">
         <v>Finance</v>
       </c>
-      <c r="G3" s="79">
+      <c r="G3" s="74">
         <v>13000</v>
       </c>
-      <c r="H3" s="79" t="str">
+      <c r="H3" s="74" t="str">
         <v>Bhopal</v>
       </c>
-      <c r="I3" s="106">
+      <c r="I3" s="101">
         <v>8569741235</v>
       </c>
       <c r="J3" s="12"/>
     </row>
     <row r="4" spans="2:10" ht="14.25" customHeight="1">
-      <c r="B4" s="65">
+      <c r="B4" s="64">
         <v>20013</v>
       </c>
-      <c r="I4" s="55"/>
+      <c r="I4" s="54"/>
     </row>
     <row r="5" spans="2:10" ht="14.25" customHeight="1" thickBot="1">
-      <c r="B5" s="57"/>
-      <c r="C5" s="58"/>
-      <c r="D5" s="58"/>
-      <c r="E5" s="58"/>
-      <c r="F5" s="58"/>
-      <c r="G5" s="58"/>
-      <c r="H5" s="58"/>
-      <c r="I5" s="60"/>
+      <c r="B5" s="56"/>
+      <c r="C5" s="57"/>
+      <c r="D5" s="57"/>
+      <c r="E5" s="57"/>
+      <c r="F5" s="57"/>
+      <c r="G5" s="57"/>
+      <c r="H5" s="57"/>
+      <c r="I5" s="59"/>
     </row>
     <row r="6" spans="2:10" ht="14.25" customHeight="1">
-      <c r="B6" s="115" t="s">
-        <v>105</v>
-      </c>
-      <c r="C6" s="55">
+      <c r="B6" s="110" t="s">
+        <v>88</v>
+      </c>
+      <c r="C6" s="54">
         <f>VLOOKUP(B7,Vlookup!B3:H15,MATCH(' hlookup(employee_table)'!B8,Vlookup!B3:H3,0),0)</f>
         <v>25500</v>
       </c>
     </row>
     <row r="7" spans="2:10">
-      <c r="B7" s="65" t="s">
+      <c r="B7" s="64" t="s">
         <v>27</v>
       </c>
-      <c r="C7" s="55"/>
+      <c r="C7" s="54"/>
     </row>
     <row r="8" spans="2:10">
-      <c r="B8" s="116" t="s">
+      <c r="B8" s="111" t="s">
         <v>6</v>
       </c>
-      <c r="C8" s="55"/>
+      <c r="C8" s="54"/>
     </row>
     <row r="9" spans="2:10" ht="15" thickBot="1">
-      <c r="B9" s="57"/>
-      <c r="C9" s="60"/>
+      <c r="B9" s="56"/>
+      <c r="C9" s="59"/>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.511811023622047" footer="0.511811023622047"/>
@@ -3577,16 +3514,16 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:11" ht="14.25" customHeight="1">
-      <c r="A1" s="129" t="s">
+      <c r="A1" s="125" t="s">
         <v>0</v>
       </c>
-      <c r="B1" s="129"/>
-      <c r="C1" s="129"/>
-      <c r="D1" s="129"/>
-      <c r="E1" s="129"/>
-      <c r="F1" s="129"/>
-      <c r="G1" s="129"/>
-      <c r="H1" s="129"/>
+      <c r="B1" s="125"/>
+      <c r="C1" s="125"/>
+      <c r="D1" s="125"/>
+      <c r="E1" s="125"/>
+      <c r="F1" s="125"/>
+      <c r="G1" s="125"/>
+      <c r="H1" s="125"/>
       <c r="J1" s="1" t="s">
         <v>36</v>
       </c>
@@ -3595,14 +3532,14 @@
       </c>
     </row>
     <row r="2" spans="1:11" ht="14.25" customHeight="1">
-      <c r="A2" s="129"/>
-      <c r="B2" s="129"/>
-      <c r="C2" s="129"/>
-      <c r="D2" s="129"/>
-      <c r="E2" s="129"/>
-      <c r="F2" s="129"/>
-      <c r="G2" s="129"/>
-      <c r="H2" s="129"/>
+      <c r="A2" s="125"/>
+      <c r="B2" s="125"/>
+      <c r="C2" s="125"/>
+      <c r="D2" s="125"/>
+      <c r="E2" s="125"/>
+      <c r="F2" s="125"/>
+      <c r="G2" s="125"/>
+      <c r="H2" s="125"/>
       <c r="J2" s="9" t="s">
         <v>60</v>
       </c>
@@ -4028,619 +3965,619 @@
   </cols>
   <sheetData>
     <row r="3" spans="2:26" ht="23.25" customHeight="1">
-      <c r="B3" s="41" t="s">
+      <c r="B3" s="40" t="s">
         <v>1</v>
       </c>
-      <c r="C3" s="41" t="s">
+      <c r="C3" s="40" t="s">
         <v>2</v>
       </c>
-      <c r="D3" s="41" t="s">
+      <c r="D3" s="40" t="s">
         <v>4</v>
       </c>
-      <c r="E3" s="41" t="s">
+      <c r="E3" s="40" t="s">
         <v>5</v>
       </c>
-      <c r="F3" s="41" t="s">
+      <c r="F3" s="40" t="s">
         <v>6</v>
       </c>
-      <c r="G3" s="41" t="s">
+      <c r="G3" s="40" t="s">
         <v>7</v>
       </c>
-      <c r="H3" s="41" t="s">
+      <c r="H3" s="40" t="s">
         <v>8</v>
       </c>
-      <c r="I3" s="45"/>
-      <c r="J3" s="22"/>
-      <c r="K3" s="41" t="s">
+      <c r="I3" s="44"/>
+      <c r="J3" s="21"/>
+      <c r="K3" s="40" t="s">
         <v>2</v>
       </c>
-      <c r="L3" s="41" t="s">
+      <c r="L3" s="40" t="s">
         <v>3</v>
       </c>
-      <c r="M3" s="41" t="s">
+      <c r="M3" s="40" t="s">
         <v>4</v>
       </c>
-      <c r="N3" s="41" t="s">
+      <c r="N3" s="40" t="s">
         <v>5</v>
       </c>
-      <c r="O3" s="41" t="s">
+      <c r="O3" s="40" t="s">
         <v>6</v>
       </c>
-      <c r="P3" s="41" t="s">
+      <c r="P3" s="40" t="s">
         <v>7</v>
       </c>
-      <c r="Q3" s="41" t="s">
+      <c r="Q3" s="40" t="s">
         <v>8</v>
       </c>
-      <c r="T3" s="52" t="s">
+      <c r="T3" s="51" t="s">
         <v>66</v>
       </c>
-      <c r="U3" s="47"/>
-      <c r="V3" s="32">
+      <c r="U3" s="46"/>
+      <c r="V3" s="31">
         <f>VLOOKUP(B7,CHOOSE({1,2},B3:B15,L3:L15),2,0)</f>
         <v>27</v>
       </c>
-      <c r="W3" s="23"/>
-      <c r="X3" s="23"/>
-      <c r="Y3" s="23"/>
-      <c r="Z3" s="24"/>
+      <c r="W3" s="22"/>
+      <c r="X3" s="22"/>
+      <c r="Y3" s="22"/>
+      <c r="Z3" s="23"/>
     </row>
     <row r="4" spans="2:26" ht="21" customHeight="1">
-      <c r="B4" s="43">
+      <c r="B4" s="42">
         <v>20012</v>
       </c>
-      <c r="C4" s="42" t="s">
+      <c r="C4" s="41" t="s">
         <v>9</v>
       </c>
-      <c r="D4" s="43" t="s">
+      <c r="D4" s="42" t="s">
         <v>10</v>
       </c>
-      <c r="E4" s="43" t="s">
+      <c r="E4" s="42" t="s">
         <v>11</v>
       </c>
-      <c r="F4" s="43">
+      <c r="F4" s="42">
         <v>26500</v>
       </c>
-      <c r="G4" s="43" t="s">
+      <c r="G4" s="42" t="s">
         <v>12</v>
       </c>
-      <c r="H4" s="44">
+      <c r="H4" s="43">
         <v>8877456987</v>
       </c>
       <c r="I4" s="19"/>
-      <c r="J4" s="21"/>
-      <c r="K4" s="42" t="s">
+      <c r="J4" s="20"/>
+      <c r="K4" s="41" t="s">
         <v>9</v>
       </c>
-      <c r="L4" s="42">
+      <c r="L4" s="41">
         <v>26</v>
       </c>
-      <c r="M4" s="43" t="s">
+      <c r="M4" s="42" t="s">
         <v>10</v>
       </c>
-      <c r="N4" s="43" t="s">
+      <c r="N4" s="42" t="s">
         <v>11</v>
       </c>
-      <c r="O4" s="43">
+      <c r="O4" s="42">
         <v>26500</v>
       </c>
-      <c r="P4" s="43" t="s">
+      <c r="P4" s="42" t="s">
         <v>12</v>
       </c>
-      <c r="Q4" s="44">
+      <c r="Q4" s="43">
         <v>8877456987</v>
       </c>
-      <c r="T4" s="27"/>
-      <c r="U4" s="28"/>
-      <c r="V4" s="28"/>
-      <c r="W4" s="28"/>
-      <c r="X4" s="28"/>
-      <c r="Y4" s="28"/>
-      <c r="Z4" s="29"/>
+      <c r="T4" s="26"/>
+      <c r="U4" s="27"/>
+      <c r="V4" s="27"/>
+      <c r="W4" s="27"/>
+      <c r="X4" s="27"/>
+      <c r="Y4" s="27"/>
+      <c r="Z4" s="28"/>
     </row>
     <row r="5" spans="2:26" ht="21" customHeight="1">
-      <c r="B5" s="43">
+      <c r="B5" s="42">
         <v>20013</v>
       </c>
-      <c r="C5" s="42" t="s">
+      <c r="C5" s="41" t="s">
         <v>13</v>
       </c>
-      <c r="D5" s="43" t="s">
+      <c r="D5" s="42" t="s">
         <v>14</v>
       </c>
-      <c r="E5" s="43" t="s">
+      <c r="E5" s="42" t="s">
         <v>15</v>
       </c>
-      <c r="F5" s="43">
+      <c r="F5" s="42">
         <v>13000</v>
       </c>
-      <c r="G5" s="43" t="s">
+      <c r="G5" s="42" t="s">
         <v>16</v>
       </c>
-      <c r="H5" s="44">
+      <c r="H5" s="43">
         <v>8569741235</v>
       </c>
       <c r="I5" s="19"/>
-      <c r="J5" s="21"/>
-      <c r="K5" s="42" t="s">
+      <c r="J5" s="20"/>
+      <c r="K5" s="41" t="s">
         <v>13</v>
       </c>
-      <c r="L5" s="42">
+      <c r="L5" s="41">
         <v>25</v>
       </c>
-      <c r="M5" s="43" t="s">
+      <c r="M5" s="42" t="s">
         <v>14</v>
       </c>
-      <c r="N5" s="43" t="s">
+      <c r="N5" s="42" t="s">
         <v>15</v>
       </c>
-      <c r="O5" s="43">
+      <c r="O5" s="42">
         <v>13000</v>
       </c>
-      <c r="P5" s="43" t="s">
+      <c r="P5" s="42" t="s">
         <v>16</v>
       </c>
-      <c r="Q5" s="44">
+      <c r="Q5" s="43">
         <v>8569741235</v>
       </c>
-      <c r="T5" s="37" t="s">
+      <c r="T5" s="36" t="s">
         <v>68</v>
       </c>
-      <c r="U5" s="30"/>
-      <c r="V5" s="33">
+      <c r="U5" s="29"/>
+      <c r="V5" s="32">
         <f>VLOOKUP(VLOOKUP(B4,B3:H15,2,0),K3:Q15,2,0)</f>
         <v>26</v>
       </c>
-      <c r="W5" s="30"/>
-      <c r="X5" s="30"/>
-      <c r="Y5" s="30"/>
-      <c r="Z5" s="31"/>
+      <c r="W5" s="29"/>
+      <c r="X5" s="29"/>
+      <c r="Y5" s="29"/>
+      <c r="Z5" s="30"/>
     </row>
     <row r="6" spans="2:26" ht="21" customHeight="1">
-      <c r="B6" s="43">
+      <c r="B6" s="42">
         <v>20014</v>
       </c>
-      <c r="C6" s="42" t="s">
+      <c r="C6" s="41" t="s">
         <v>17</v>
       </c>
-      <c r="D6" s="43" t="s">
+      <c r="D6" s="42" t="s">
         <v>18</v>
       </c>
-      <c r="E6" s="43" t="s">
+      <c r="E6" s="42" t="s">
         <v>11</v>
       </c>
-      <c r="F6" s="43">
+      <c r="F6" s="42">
         <v>20000</v>
       </c>
-      <c r="G6" s="43" t="s">
+      <c r="G6" s="42" t="s">
         <v>12</v>
       </c>
-      <c r="H6" s="44">
+      <c r="H6" s="43">
         <v>7584963214</v>
       </c>
       <c r="I6" s="19"/>
-      <c r="J6" s="21"/>
-      <c r="K6" s="42" t="s">
+      <c r="J6" s="20"/>
+      <c r="K6" s="41" t="s">
         <v>17</v>
       </c>
-      <c r="L6" s="42">
+      <c r="L6" s="41">
         <v>28</v>
       </c>
-      <c r="M6" s="43" t="s">
+      <c r="M6" s="42" t="s">
         <v>18</v>
       </c>
-      <c r="N6" s="43" t="s">
+      <c r="N6" s="42" t="s">
         <v>11</v>
       </c>
-      <c r="O6" s="43">
+      <c r="O6" s="42">
         <v>20000</v>
       </c>
-      <c r="P6" s="43" t="s">
+      <c r="P6" s="42" t="s">
         <v>12</v>
       </c>
-      <c r="Q6" s="44">
+      <c r="Q6" s="43">
         <v>7584963214</v>
       </c>
-      <c r="T6" s="46" t="s">
+      <c r="T6" s="45" t="s">
         <v>69</v>
       </c>
-      <c r="U6" s="47"/>
-      <c r="V6" s="47"/>
-      <c r="W6" s="47"/>
-      <c r="X6" s="47"/>
-      <c r="Y6" s="47"/>
-      <c r="Z6" s="48"/>
+      <c r="U6" s="46"/>
+      <c r="V6" s="46"/>
+      <c r="W6" s="46"/>
+      <c r="X6" s="46"/>
+      <c r="Y6" s="46"/>
+      <c r="Z6" s="47"/>
     </row>
     <row r="7" spans="2:26" ht="21" customHeight="1">
-      <c r="B7" s="43">
+      <c r="B7" s="42">
         <v>20015</v>
       </c>
-      <c r="C7" s="42" t="s">
+      <c r="C7" s="41" t="s">
         <v>19</v>
       </c>
-      <c r="D7" s="43" t="s">
+      <c r="D7" s="42" t="s">
         <v>14</v>
       </c>
-      <c r="E7" s="43" t="s">
+      <c r="E7" s="42" t="s">
         <v>15</v>
       </c>
-      <c r="F7" s="43">
+      <c r="F7" s="42">
         <v>15000</v>
       </c>
-      <c r="G7" s="43" t="s">
+      <c r="G7" s="42" t="s">
         <v>16</v>
       </c>
-      <c r="H7" s="44">
+      <c r="H7" s="43">
         <v>7788994455</v>
       </c>
       <c r="I7" s="19"/>
-      <c r="J7" s="21"/>
-      <c r="K7" s="42" t="s">
+      <c r="J7" s="20"/>
+      <c r="K7" s="41" t="s">
         <v>19</v>
       </c>
-      <c r="L7" s="42">
+      <c r="L7" s="41">
         <v>27</v>
       </c>
-      <c r="M7" s="43" t="s">
+      <c r="M7" s="42" t="s">
         <v>14</v>
       </c>
-      <c r="N7" s="43" t="s">
+      <c r="N7" s="42" t="s">
         <v>15</v>
       </c>
-      <c r="O7" s="43">
+      <c r="O7" s="42">
         <v>15000</v>
       </c>
-      <c r="P7" s="43" t="s">
+      <c r="P7" s="42" t="s">
         <v>16</v>
       </c>
-      <c r="Q7" s="44">
+      <c r="Q7" s="43">
         <v>7788994455</v>
       </c>
-      <c r="T7" s="27"/>
-      <c r="U7" s="34" cm="1">
+      <c r="T7" s="26"/>
+      <c r="U7" s="33" cm="1">
         <f t="array" ref="U7:Z7">VLOOKUP(VLOOKUP(B4,B3:H15,2,0),K3:Q15,{2,3,4,5,6,7},0)</f>
         <v>26</v>
       </c>
-      <c r="V7" s="34" t="str">
+      <c r="V7" s="33" t="str">
         <v>Engineer</v>
       </c>
-      <c r="W7" s="34" t="str">
+      <c r="W7" s="33" t="str">
         <v>Technical</v>
       </c>
-      <c r="X7" s="34">
+      <c r="X7" s="33">
         <v>26500</v>
       </c>
-      <c r="Y7" s="34" t="str">
+      <c r="Y7" s="33" t="str">
         <v>Indore</v>
       </c>
-      <c r="Z7" s="35">
+      <c r="Z7" s="34">
         <v>8877456987</v>
       </c>
     </row>
     <row r="8" spans="2:26" ht="21" customHeight="1">
-      <c r="B8" s="43">
+      <c r="B8" s="42">
         <v>20016</v>
       </c>
-      <c r="C8" s="42" t="s">
+      <c r="C8" s="41" t="s">
         <v>20</v>
       </c>
-      <c r="D8" s="43" t="s">
+      <c r="D8" s="42" t="s">
         <v>10</v>
       </c>
-      <c r="E8" s="43" t="s">
+      <c r="E8" s="42" t="s">
         <v>11</v>
       </c>
-      <c r="F8" s="43">
+      <c r="F8" s="42">
         <v>20000</v>
       </c>
-      <c r="G8" s="43" t="s">
+      <c r="G8" s="42" t="s">
         <v>21</v>
       </c>
-      <c r="H8" s="44">
+      <c r="H8" s="43">
         <v>8798654512</v>
       </c>
       <c r="I8" s="19"/>
-      <c r="J8" s="21"/>
-      <c r="K8" s="42" t="s">
+      <c r="J8" s="20"/>
+      <c r="K8" s="41" t="s">
         <v>20</v>
       </c>
-      <c r="L8" s="42">
+      <c r="L8" s="41">
         <v>25</v>
       </c>
-      <c r="M8" s="43" t="s">
+      <c r="M8" s="42" t="s">
         <v>10</v>
       </c>
-      <c r="N8" s="43" t="s">
+      <c r="N8" s="42" t="s">
         <v>11</v>
       </c>
-      <c r="O8" s="43">
+      <c r="O8" s="42">
         <v>20000</v>
       </c>
-      <c r="P8" s="43" t="s">
+      <c r="P8" s="42" t="s">
         <v>21</v>
       </c>
-      <c r="Q8" s="44">
+      <c r="Q8" s="43">
         <v>8798654512</v>
       </c>
-      <c r="T8" s="25"/>
-      <c r="Z8" s="26"/>
+      <c r="T8" s="24"/>
+      <c r="Z8" s="25"/>
     </row>
     <row r="9" spans="2:26" ht="21" customHeight="1">
-      <c r="B9" s="43">
+      <c r="B9" s="42">
         <v>20017</v>
       </c>
-      <c r="C9" s="42" t="s">
+      <c r="C9" s="41" t="s">
         <v>22</v>
       </c>
-      <c r="D9" s="43" t="s">
+      <c r="D9" s="42" t="s">
         <v>10</v>
       </c>
-      <c r="E9" s="43" t="s">
+      <c r="E9" s="42" t="s">
         <v>11</v>
       </c>
-      <c r="F9" s="43">
+      <c r="F9" s="42">
         <v>33000</v>
       </c>
-      <c r="G9" s="43" t="s">
+      <c r="G9" s="42" t="s">
         <v>16</v>
       </c>
-      <c r="H9" s="44">
+      <c r="H9" s="43">
         <v>9874563214</v>
       </c>
       <c r="I9" s="19"/>
-      <c r="J9" s="21"/>
-      <c r="K9" s="42" t="s">
+      <c r="J9" s="20"/>
+      <c r="K9" s="41" t="s">
         <v>22</v>
       </c>
-      <c r="L9" s="42">
+      <c r="L9" s="41">
         <v>26</v>
       </c>
-      <c r="M9" s="43" t="s">
+      <c r="M9" s="42" t="s">
         <v>10</v>
       </c>
-      <c r="N9" s="43" t="s">
+      <c r="N9" s="42" t="s">
         <v>11</v>
       </c>
-      <c r="O9" s="43">
+      <c r="O9" s="42">
         <v>33000</v>
       </c>
-      <c r="P9" s="43" t="s">
+      <c r="P9" s="42" t="s">
         <v>16</v>
       </c>
-      <c r="Q9" s="44">
+      <c r="Q9" s="43">
         <v>9874563214</v>
       </c>
-      <c r="T9" s="49" t="s">
+      <c r="T9" s="48" t="s">
         <v>71</v>
       </c>
       <c r="U9" s="2"/>
       <c r="V9" s="2"/>
-      <c r="W9" s="36" t="str">
+      <c r="W9" s="35" t="str">
         <f>IFERROR(VLOOKUP(VLOOKUP(B5,B3:H15,2,0),K3:Q15,MATCH(V11,K3:Q3,0),0),"Not available")</f>
         <v>Accountant</v>
       </c>
-      <c r="Z9" s="26"/>
+      <c r="Z9" s="25"/>
     </row>
     <row r="10" spans="2:26" ht="21" customHeight="1">
-      <c r="B10" s="43">
+      <c r="B10" s="42">
         <v>20018</v>
       </c>
-      <c r="C10" s="42" t="s">
+      <c r="C10" s="41" t="s">
         <v>23</v>
       </c>
-      <c r="D10" s="43" t="s">
+      <c r="D10" s="42" t="s">
         <v>18</v>
       </c>
-      <c r="E10" s="43" t="s">
+      <c r="E10" s="42" t="s">
         <v>11</v>
       </c>
-      <c r="F10" s="43">
+      <c r="F10" s="42">
         <v>21000</v>
       </c>
-      <c r="G10" s="43" t="s">
+      <c r="G10" s="42" t="s">
         <v>12</v>
       </c>
-      <c r="H10" s="44">
+      <c r="H10" s="43">
         <v>8974563214</v>
       </c>
       <c r="I10" s="19"/>
-      <c r="J10" s="21"/>
-      <c r="K10" s="42" t="s">
+      <c r="J10" s="20"/>
+      <c r="K10" s="41" t="s">
         <v>23</v>
       </c>
-      <c r="L10" s="42">
+      <c r="L10" s="41">
         <v>25</v>
       </c>
-      <c r="M10" s="43" t="s">
+      <c r="M10" s="42" t="s">
         <v>18</v>
       </c>
-      <c r="N10" s="43" t="s">
+      <c r="N10" s="42" t="s">
         <v>11</v>
       </c>
-      <c r="O10" s="43">
+      <c r="O10" s="42">
         <v>21000</v>
       </c>
-      <c r="P10" s="43" t="s">
+      <c r="P10" s="42" t="s">
         <v>12</v>
       </c>
-      <c r="Q10" s="44">
+      <c r="Q10" s="43">
         <v>8974563214</v>
       </c>
-      <c r="T10" s="27"/>
-      <c r="U10" s="28"/>
-      <c r="V10" s="28"/>
-      <c r="W10" s="28"/>
-      <c r="X10" s="28"/>
-      <c r="Y10" s="28"/>
-      <c r="Z10" s="29"/>
+      <c r="T10" s="26"/>
+      <c r="U10" s="27"/>
+      <c r="V10" s="27"/>
+      <c r="W10" s="27"/>
+      <c r="X10" s="27"/>
+      <c r="Y10" s="27"/>
+      <c r="Z10" s="28"/>
     </row>
     <row r="11" spans="2:26" ht="15.5">
-      <c r="B11" s="43">
+      <c r="B11" s="42">
         <v>20019</v>
       </c>
-      <c r="C11" s="42" t="s">
+      <c r="C11" s="41" t="s">
         <v>24</v>
       </c>
-      <c r="D11" s="43" t="s">
+      <c r="D11" s="42" t="s">
         <v>14</v>
       </c>
-      <c r="E11" s="43" t="s">
+      <c r="E11" s="42" t="s">
         <v>15</v>
       </c>
-      <c r="F11" s="43">
+      <c r="F11" s="42">
         <v>31500</v>
       </c>
-      <c r="G11" s="43" t="s">
+      <c r="G11" s="42" t="s">
         <v>16</v>
       </c>
-      <c r="H11" s="44">
+      <c r="H11" s="43">
         <v>8745968745</v>
       </c>
       <c r="I11" s="19"/>
-      <c r="J11" s="21"/>
-      <c r="K11" s="42" t="s">
+      <c r="J11" s="20"/>
+      <c r="K11" s="41" t="s">
         <v>24</v>
       </c>
-      <c r="L11" s="42">
+      <c r="L11" s="41">
         <v>26</v>
       </c>
-      <c r="M11" s="43" t="s">
+      <c r="M11" s="42" t="s">
         <v>14</v>
       </c>
-      <c r="N11" s="43" t="s">
+      <c r="N11" s="42" t="s">
         <v>15</v>
       </c>
-      <c r="O11" s="43">
+      <c r="O11" s="42">
         <v>31500</v>
       </c>
-      <c r="P11" s="43" t="s">
+      <c r="P11" s="42" t="s">
         <v>16</v>
       </c>
-      <c r="Q11" s="44">
+      <c r="Q11" s="43">
         <v>8745968745</v>
       </c>
-      <c r="T11" s="39" t="s">
+      <c r="T11" s="38" t="s">
         <v>65</v>
       </c>
-      <c r="U11" s="50">
+      <c r="U11" s="49">
         <v>20019</v>
       </c>
-      <c r="V11" s="51" t="s">
+      <c r="V11" s="50" t="s">
         <v>4</v>
       </c>
-      <c r="W11" s="23"/>
-      <c r="X11" s="23"/>
-      <c r="Y11" s="23"/>
-      <c r="Z11" s="24"/>
+      <c r="W11" s="22"/>
+      <c r="X11" s="22"/>
+      <c r="Y11" s="22"/>
+      <c r="Z11" s="23"/>
     </row>
     <row r="12" spans="2:26" ht="21" customHeight="1">
-      <c r="B12" s="43">
+      <c r="B12" s="42">
         <v>20020</v>
       </c>
-      <c r="C12" s="42" t="s">
+      <c r="C12" s="41" t="s">
         <v>26</v>
       </c>
-      <c r="D12" s="43" t="s">
+      <c r="D12" s="42" t="s">
         <v>14</v>
       </c>
-      <c r="E12" s="43" t="s">
+      <c r="E12" s="42" t="s">
         <v>15</v>
       </c>
-      <c r="F12" s="43">
+      <c r="F12" s="42">
         <v>40500</v>
       </c>
-      <c r="G12" s="43" t="s">
+      <c r="G12" s="42" t="s">
         <v>12</v>
       </c>
-      <c r="H12" s="44">
+      <c r="H12" s="43">
         <v>9874569874</v>
       </c>
       <c r="I12" s="19"/>
-      <c r="J12" s="21"/>
-      <c r="K12" s="42" t="s">
+      <c r="J12" s="20"/>
+      <c r="K12" s="41" t="s">
         <v>26</v>
       </c>
-      <c r="L12" s="42">
+      <c r="L12" s="41">
         <v>28</v>
       </c>
-      <c r="M12" s="43" t="s">
+      <c r="M12" s="42" t="s">
         <v>14</v>
       </c>
-      <c r="N12" s="43" t="s">
+      <c r="N12" s="42" t="s">
         <v>15</v>
       </c>
-      <c r="O12" s="43">
+      <c r="O12" s="42">
         <v>40500</v>
       </c>
-      <c r="P12" s="43" t="s">
+      <c r="P12" s="42" t="s">
         <v>12</v>
       </c>
-      <c r="Q12" s="44">
+      <c r="Q12" s="43">
         <v>9874569874</v>
       </c>
-      <c r="T12" s="38" t="s">
+      <c r="T12" s="37" t="s">
         <v>67</v>
       </c>
       <c r="V12" s="2"/>
       <c r="W12" s="2"/>
       <c r="X12" s="2"/>
-      <c r="Z12" s="26"/>
+      <c r="Z12" s="25"/>
     </row>
     <row r="13" spans="2:26" ht="21" customHeight="1">
-      <c r="B13" s="43">
+      <c r="B13" s="42">
         <v>20021</v>
       </c>
-      <c r="C13" s="42" t="s">
+      <c r="C13" s="41" t="s">
         <v>27</v>
       </c>
-      <c r="D13" s="43" t="s">
+      <c r="D13" s="42" t="s">
         <v>10</v>
       </c>
-      <c r="E13" s="43" t="s">
+      <c r="E13" s="42" t="s">
         <v>11</v>
       </c>
-      <c r="F13" s="43">
+      <c r="F13" s="42">
         <v>25500</v>
       </c>
-      <c r="G13" s="43" t="s">
+      <c r="G13" s="42" t="s">
         <v>21</v>
       </c>
-      <c r="H13" s="44">
+      <c r="H13" s="43">
         <v>8574965874</v>
       </c>
       <c r="I13" s="19"/>
-      <c r="J13" s="21"/>
-      <c r="K13" s="42" t="s">
+      <c r="J13" s="20"/>
+      <c r="K13" s="41" t="s">
         <v>27</v>
       </c>
-      <c r="L13" s="42">
+      <c r="L13" s="41">
         <v>27</v>
       </c>
-      <c r="M13" s="43" t="s">
+      <c r="M13" s="42" t="s">
         <v>10</v>
       </c>
-      <c r="N13" s="43" t="s">
+      <c r="N13" s="42" t="s">
         <v>11</v>
       </c>
-      <c r="O13" s="43">
+      <c r="O13" s="42">
         <v>25500</v>
       </c>
-      <c r="P13" s="43" t="s">
+      <c r="P13" s="42" t="s">
         <v>21</v>
       </c>
-      <c r="Q13" s="44">
+      <c r="Q13" s="43">
         <v>8574965874</v>
       </c>
-      <c r="T13" s="27"/>
-      <c r="U13" s="28"/>
-      <c r="V13" s="34" t="str">
+      <c r="T13" s="26"/>
+      <c r="U13" s="27"/>
+      <c r="V13" s="33" t="str">
         <f>VLOOKUP(VLOOKUP(U11,B3:H15,2,0),K3:Q15,MATCH(V11,K3:Q3,0),0)</f>
         <v>Accountant</v>
       </c>
-      <c r="W13" s="28"/>
-      <c r="X13" s="28"/>
-      <c r="Y13" s="28"/>
-      <c r="Z13" s="29"/>
+      <c r="W13" s="27"/>
+      <c r="X13" s="27"/>
+      <c r="Y13" s="27"/>
+      <c r="Z13" s="28"/>
     </row>
     <row r="14" spans="2:26">
       <c r="B14" s="16">
@@ -4685,18 +4622,18 @@
       <c r="Q14" s="15">
         <v>8521479632</v>
       </c>
-      <c r="T14" s="40" t="s">
+      <c r="T14" s="39" t="s">
         <v>70</v>
       </c>
-      <c r="U14" s="23"/>
-      <c r="V14" s="32" t="str">
+      <c r="U14" s="22"/>
+      <c r="V14" s="31" t="str">
         <f>IFERROR(VLOOKUP(B5,B3:H15,8,0),"not available")</f>
         <v>not available</v>
       </c>
-      <c r="W14" s="23"/>
-      <c r="X14" s="23"/>
-      <c r="Y14" s="23"/>
-      <c r="Z14" s="24"/>
+      <c r="W14" s="22"/>
+      <c r="X14" s="22"/>
+      <c r="Y14" s="22"/>
+      <c r="Z14" s="23"/>
     </row>
     <row r="15" spans="2:26" ht="21" customHeight="1">
       <c r="B15" s="16">
@@ -4741,13 +4678,13 @@
       <c r="Q15" s="15">
         <v>8569745623</v>
       </c>
-      <c r="T15" s="27"/>
-      <c r="U15" s="28"/>
-      <c r="V15" s="28"/>
-      <c r="W15" s="28"/>
-      <c r="X15" s="28"/>
-      <c r="Y15" s="28"/>
-      <c r="Z15" s="29"/>
+      <c r="T15" s="26"/>
+      <c r="U15" s="27"/>
+      <c r="V15" s="27"/>
+      <c r="W15" s="27"/>
+      <c r="X15" s="27"/>
+      <c r="Y15" s="27"/>
+      <c r="Z15" s="28"/>
     </row>
     <row r="17" spans="10:12" ht="18" customHeight="1"/>
     <row r="18" spans="10:12" ht="54.75" customHeight="1"/>
@@ -4755,9 +4692,9 @@
     <row r="20" spans="10:12" ht="14.25" customHeight="1"/>
     <row r="21" spans="10:12" ht="27.75" customHeight="1"/>
     <row r="22" spans="10:12" ht="36" customHeight="1">
-      <c r="J22" s="134"/>
-      <c r="K22" s="134"/>
-      <c r="L22" s="134"/>
+      <c r="J22" s="130"/>
+      <c r="K22" s="130"/>
+      <c r="L22" s="130"/>
     </row>
     <row r="24" spans="10:12" ht="41.25" customHeight="1"/>
     <row r="25" spans="10:12" ht="14.25" customHeight="1"/>
@@ -4888,11 +4825,11 @@
       <c r="O2" s="5">
         <v>8877456987</v>
       </c>
-      <c r="Q2" s="62" t="s">
+      <c r="Q2" s="61" t="s">
         <v>72</v>
       </c>
-      <c r="R2" s="53"/>
-      <c r="S2" s="54">
+      <c r="R2" s="52"/>
+      <c r="S2" s="53">
         <f>VLOOKUP(VLOOKUP(R3,CHOOSE({1,2},B1:B13,A1:A13),2,0),I1:O13,2,0)</f>
         <v>25</v>
       </c>
@@ -4943,13 +4880,13 @@
       <c r="O3" s="5">
         <v>8569741235</v>
       </c>
-      <c r="Q3" s="61" t="s">
+      <c r="Q3" s="60" t="s">
         <v>73</v>
       </c>
-      <c r="R3" s="63">
+      <c r="R3" s="62">
         <v>20013</v>
       </c>
-      <c r="S3" s="55"/>
+      <c r="S3" s="54"/>
     </row>
     <row r="4" spans="1:22" ht="21" customHeight="1" thickBot="1">
       <c r="A4" s="4" t="s">
@@ -4994,9 +4931,9 @@
       <c r="O4" s="5">
         <v>7584963214</v>
       </c>
-      <c r="Q4" s="57"/>
-      <c r="R4" s="58"/>
-      <c r="S4" s="60"/>
+      <c r="Q4" s="56"/>
+      <c r="R4" s="57"/>
+      <c r="S4" s="59"/>
     </row>
     <row r="5" spans="1:22" ht="21" customHeight="1">
       <c r="A5" s="4" t="s">
@@ -5041,11 +4978,11 @@
       <c r="O5" s="5">
         <v>7788994455</v>
       </c>
-      <c r="Q5" s="135" t="s">
+      <c r="Q5" s="131" t="s">
         <v>74</v>
       </c>
-      <c r="R5" s="136"/>
-      <c r="S5" s="137"/>
+      <c r="R5" s="132"/>
+      <c r="S5" s="133"/>
     </row>
     <row r="6" spans="1:22" ht="21" customHeight="1" thickBot="1">
       <c r="A6" s="4" t="s">
@@ -5090,14 +5027,14 @@
       <c r="O6" s="5">
         <v>8798654512</v>
       </c>
-      <c r="Q6" s="57">
+      <c r="Q6" s="56">
         <f t="array" ref="Q6:S6">IFERROR(VLOOKUP(VLOOKUP(R3,CHOOSE({1,2},B:B,A:A),2,0),I1:O13,{2,4,7},0),"NOT AVAILABLE")</f>
         <v>25</v>
       </c>
-      <c r="R6" s="58" t="str">
+      <c r="R6" s="57" t="str">
         <v>Finance</v>
       </c>
-      <c r="S6" s="59">
+      <c r="S6" s="58">
         <v>8569741235</v>
       </c>
     </row>
@@ -5430,159 +5367,6 @@
 </file>
 
 <file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0500-000000000000}">
-  <dimension ref="A1:G13"/>
-  <sheetFormatPr defaultColWidth="8.6328125" defaultRowHeight="14.5"/>
-  <cols>
-    <col min="1" max="1" width="10" customWidth="1"/>
-    <col min="2" max="2" width="8" customWidth="1"/>
-    <col min="3" max="3" width="70.26953125" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="10" customWidth="1"/>
-    <col min="6" max="6" width="68.08984375" bestFit="1" customWidth="1"/>
-    <col min="7" max="7" width="4" bestFit="1" customWidth="1"/>
-  </cols>
-  <sheetData>
-    <row r="1" spans="1:7" ht="51" customHeight="1">
-      <c r="A1" s="1" t="s">
-        <v>75</v>
-      </c>
-      <c r="B1" s="20" t="s">
-        <v>76</v>
-      </c>
-      <c r="C1" s="69" t="s">
-        <v>77</v>
-      </c>
-      <c r="D1" s="54" t="str">
-        <f>VLOOKUP(D2,A1:B6,2,1)</f>
-        <v>B</v>
-      </c>
-    </row>
-    <row r="2" spans="1:7" ht="14.25" customHeight="1" thickBot="1">
-      <c r="A2" s="3">
-        <v>0</v>
-      </c>
-      <c r="B2" s="21" t="s">
-        <v>78</v>
-      </c>
-      <c r="C2" s="67" t="s">
-        <v>79</v>
-      </c>
-      <c r="D2" s="68">
-        <v>82</v>
-      </c>
-    </row>
-    <row r="3" spans="1:7" ht="14.25" customHeight="1">
-      <c r="A3" s="3">
-        <v>40</v>
-      </c>
-      <c r="B3" s="3" t="s">
-        <v>80</v>
-      </c>
-    </row>
-    <row r="4" spans="1:7" ht="14.25" customHeight="1">
-      <c r="A4" s="3">
-        <v>60</v>
-      </c>
-      <c r="B4" s="3" t="s">
-        <v>81</v>
-      </c>
-    </row>
-    <row r="5" spans="1:7" ht="14.25" customHeight="1">
-      <c r="A5" s="3">
-        <v>75</v>
-      </c>
-      <c r="B5" s="3" t="s">
-        <v>82</v>
-      </c>
-    </row>
-    <row r="6" spans="1:7" ht="14.25" customHeight="1">
-      <c r="A6" s="3">
-        <v>90</v>
-      </c>
-      <c r="B6" s="3" t="s">
-        <v>83</v>
-      </c>
-    </row>
-    <row r="8" spans="1:7" ht="68.25" customHeight="1"/>
-    <row r="9" spans="1:7" ht="14.25" customHeight="1"/>
-    <row r="10" spans="1:7" ht="14.25" customHeight="1" thickBot="1">
-      <c r="A10" s="1" t="s">
-        <v>87</v>
-      </c>
-      <c r="B10" s="1" t="s">
-        <v>86</v>
-      </c>
-      <c r="C10" s="1" t="s">
-        <v>88</v>
-      </c>
-      <c r="D10" s="1" t="s">
-        <v>89</v>
-      </c>
-    </row>
-    <row r="11" spans="1:7">
-      <c r="A11" s="3" t="s">
-        <v>90</v>
-      </c>
-      <c r="B11" s="3">
-        <v>110</v>
-      </c>
-      <c r="C11" s="3">
-        <v>105</v>
-      </c>
-      <c r="D11" s="3">
-        <v>106</v>
-      </c>
-      <c r="F11" s="64" t="s">
-        <v>84</v>
-      </c>
-      <c r="G11" s="54">
-        <f>VLOOKUP(F12,A10:D13,MATCH(F13,A10:D10,0),0)</f>
-        <v>110</v>
-      </c>
-    </row>
-    <row r="12" spans="1:7">
-      <c r="A12" s="3" t="s">
-        <v>85</v>
-      </c>
-      <c r="B12" s="3">
-        <v>110</v>
-      </c>
-      <c r="C12" s="3">
-        <v>104</v>
-      </c>
-      <c r="D12" s="3">
-        <v>105</v>
-      </c>
-      <c r="F12" s="65" t="s">
-        <v>85</v>
-      </c>
-      <c r="G12" s="55"/>
-    </row>
-    <row r="13" spans="1:7" ht="14.25" customHeight="1" thickBot="1">
-      <c r="A13" s="3" t="s">
-        <v>91</v>
-      </c>
-      <c r="B13" s="3">
-        <v>103</v>
-      </c>
-      <c r="C13" s="3">
-        <v>100</v>
-      </c>
-      <c r="D13" s="3">
-        <v>106</v>
-      </c>
-      <c r="F13" s="66" t="s">
-        <v>86</v>
-      </c>
-      <c r="G13" s="60"/>
-    </row>
-  </sheetData>
-  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.511811023622047" footer="0.511811023622047"/>
-  <pageSetup paperSize="9" orientation="portrait" horizontalDpi="300" verticalDpi="300"/>
-</worksheet>
-</file>
-
-<file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0600-000000000000}">
   <dimension ref="B2:Q40"/>
   <sheetFormatPr defaultColWidth="8.6328125" defaultRowHeight="14.5"/>
@@ -5604,10 +5388,10 @@
   </cols>
   <sheetData>
     <row r="2" spans="3:17" ht="21" customHeight="1">
-      <c r="C2" s="138" t="s">
+      <c r="C2" s="134" t="s">
         <v>0</v>
       </c>
-      <c r="D2" s="138"/>
+      <c r="D2" s="134"/>
       <c r="E2" s="1" t="s">
         <v>1</v>
       </c>
@@ -5649,8 +5433,8 @@
       </c>
     </row>
     <row r="3" spans="3:17" ht="23.25" customHeight="1">
-      <c r="C3" s="138"/>
-      <c r="D3" s="138"/>
+      <c r="C3" s="134"/>
+      <c r="D3" s="134"/>
       <c r="E3" s="11" t="s">
         <v>2</v>
       </c>
@@ -5692,8 +5476,8 @@
       </c>
     </row>
     <row r="4" spans="3:17" ht="23.25" customHeight="1">
-      <c r="C4" s="138"/>
-      <c r="D4" s="138"/>
+      <c r="C4" s="134"/>
+      <c r="D4" s="134"/>
       <c r="E4" s="11" t="s">
         <v>3</v>
       </c>
@@ -5735,8 +5519,8 @@
       </c>
     </row>
     <row r="5" spans="3:17" ht="21" customHeight="1">
-      <c r="C5" s="138"/>
-      <c r="D5" s="138"/>
+      <c r="C5" s="134"/>
+      <c r="D5" s="134"/>
       <c r="E5" s="11" t="s">
         <v>4</v>
       </c>
@@ -5778,8 +5562,8 @@
       </c>
     </row>
     <row r="6" spans="3:17" ht="21" customHeight="1">
-      <c r="C6" s="138"/>
-      <c r="D6" s="138"/>
+      <c r="C6" s="134"/>
+      <c r="D6" s="134"/>
       <c r="E6" s="11" t="s">
         <v>5</v>
       </c>
@@ -5821,8 +5605,8 @@
       </c>
     </row>
     <row r="7" spans="3:17" ht="21" customHeight="1">
-      <c r="C7" s="138"/>
-      <c r="D7" s="138"/>
+      <c r="C7" s="134"/>
+      <c r="D7" s="134"/>
       <c r="E7" s="11" t="s">
         <v>6</v>
       </c>
@@ -5864,8 +5648,8 @@
       </c>
     </row>
     <row r="8" spans="3:17" ht="21" customHeight="1">
-      <c r="C8" s="138"/>
-      <c r="D8" s="138"/>
+      <c r="C8" s="134"/>
+      <c r="D8" s="134"/>
       <c r="E8" s="11" t="s">
         <v>7</v>
       </c>
@@ -5907,8 +5691,8 @@
       </c>
     </row>
     <row r="9" spans="3:17" ht="21" customHeight="1">
-      <c r="C9" s="138"/>
-      <c r="D9" s="138"/>
+      <c r="C9" s="134"/>
+      <c r="D9" s="134"/>
       <c r="E9" s="11" t="s">
         <v>8</v>
       </c>
@@ -5950,179 +5734,179 @@
       </c>
     </row>
     <row r="12" spans="3:17" ht="15" thickBot="1">
-      <c r="C12" s="75" t="s">
-        <v>92</v>
-      </c>
-      <c r="D12" s="76">
+      <c r="C12" s="70" t="s">
+        <v>75</v>
+      </c>
+      <c r="D12" s="71">
         <v>20014</v>
       </c>
     </row>
     <row r="13" spans="3:17" ht="36" customHeight="1" thickBot="1">
-      <c r="C13" s="73" t="s">
-        <v>93</v>
-      </c>
-      <c r="D13" s="71" t="str">
+      <c r="C13" s="68" t="s">
+        <v>76</v>
+      </c>
+      <c r="D13" s="66" t="str">
         <f>HLOOKUP(D12,C2:Q9,2,0)</f>
         <v>Kapil Singh</v>
       </c>
     </row>
     <row r="14" spans="3:17" ht="14.25" customHeight="1" thickBot="1"/>
     <row r="15" spans="3:17" ht="41.25" customHeight="1" thickBot="1">
-      <c r="C15" s="73" t="s">
-        <v>94</v>
-      </c>
-      <c r="D15" s="72" t="str">
+      <c r="C15" s="68" t="s">
+        <v>77</v>
+      </c>
+      <c r="D15" s="67" t="str">
         <f t="array" ref="D15:F15">HLOOKUP(D12,E2:Q9,{2,3,4},0)</f>
         <v>Kapil Singh</v>
       </c>
-      <c r="E15" s="72">
+      <c r="E15" s="67">
         <v>28</v>
       </c>
-      <c r="F15" s="71" t="str">
+      <c r="F15" s="66" t="str">
         <v>CAD Designer</v>
       </c>
     </row>
     <row r="16" spans="3:17" ht="14.25" customHeight="1"/>
     <row r="17" spans="3:7" ht="14.25" customHeight="1" thickBot="1"/>
     <row r="18" spans="3:7" ht="27.75" customHeight="1">
-      <c r="C18" s="74" t="s">
-        <v>95</v>
-      </c>
-      <c r="D18" s="54">
+      <c r="C18" s="69" t="s">
+        <v>78</v>
+      </c>
+      <c r="D18" s="53">
         <f>HLOOKUP(D12,E2:Q9,MATCH(C19,E2:E9,0),0)</f>
         <v>20000</v>
       </c>
-      <c r="E18" s="70"/>
-      <c r="F18" s="70"/>
+      <c r="E18" s="65"/>
+      <c r="F18" s="65"/>
     </row>
     <row r="19" spans="3:7" ht="14.25" customHeight="1" thickBot="1">
-      <c r="C19" s="77" t="s">
+      <c r="C19" s="72" t="s">
         <v>6</v>
       </c>
-      <c r="D19" s="60"/>
+      <c r="D19" s="59"/>
     </row>
     <row r="20" spans="3:7" ht="14.25" customHeight="1"/>
     <row r="21" spans="3:7" ht="14.25" customHeight="1"/>
     <row r="22" spans="3:7" ht="14.25" customHeight="1" thickBot="1"/>
     <row r="23" spans="3:7" ht="14.25" customHeight="1">
-      <c r="C23" s="74" t="s">
-        <v>96</v>
-      </c>
-      <c r="D23" s="54" t="str">
+      <c r="C23" s="69" t="s">
+        <v>79</v>
+      </c>
+      <c r="D23" s="53" t="str">
         <f>HLOOKUP($D$12,$E$2:$Q$9,ROWS($E$2:E3),0)</f>
         <v>Kapil Singh</v>
       </c>
-      <c r="E23" s="70"/>
-      <c r="F23" s="70"/>
-      <c r="G23" s="70"/>
+      <c r="E23" s="65"/>
+      <c r="F23" s="65"/>
+      <c r="G23" s="65"/>
     </row>
     <row r="24" spans="3:7" ht="14.25" customHeight="1">
-      <c r="C24" s="56"/>
-      <c r="D24" s="55">
+      <c r="C24" s="55"/>
+      <c r="D24" s="54">
         <f>HLOOKUP($D$12,$E$2:$Q$9,ROWS($E$2:E4),0)</f>
         <v>28</v>
       </c>
     </row>
     <row r="25" spans="3:7" ht="14.25" customHeight="1">
-      <c r="C25" s="56"/>
-      <c r="D25" s="55" t="str">
+      <c r="C25" s="55"/>
+      <c r="D25" s="54" t="str">
         <f>HLOOKUP($D$12,$E$2:$Q$9,ROWS($E$2:E5),0)</f>
         <v>CAD Designer</v>
       </c>
     </row>
     <row r="26" spans="3:7" ht="27.75" customHeight="1">
-      <c r="C26" s="56"/>
-      <c r="D26" s="55" t="str">
+      <c r="C26" s="55"/>
+      <c r="D26" s="54" t="str">
         <f>HLOOKUP($D$12,$E$2:$Q$9,ROWS($E$2:E6),0)</f>
         <v>Technical</v>
       </c>
     </row>
     <row r="27" spans="3:7" ht="14.25" customHeight="1">
-      <c r="C27" s="56"/>
-      <c r="D27" s="55">
+      <c r="C27" s="55"/>
+      <c r="D27" s="54">
         <f>HLOOKUP($D$12,$E$2:$Q$9,ROWS($E$2:E7),0)</f>
         <v>20000</v>
       </c>
     </row>
     <row r="28" spans="3:7" ht="14.25" customHeight="1">
-      <c r="C28" s="56"/>
-      <c r="D28" s="55" t="str">
+      <c r="C28" s="55"/>
+      <c r="D28" s="54" t="str">
         <f>HLOOKUP($D$12,$E$2:$Q$9,ROWS($E$2:E8),0)</f>
         <v>Indore</v>
       </c>
     </row>
     <row r="29" spans="3:7" ht="14.25" customHeight="1" thickBot="1">
-      <c r="C29" s="57"/>
-      <c r="D29" s="59">
+      <c r="C29" s="56"/>
+      <c r="D29" s="58">
         <f>HLOOKUP($D$12,$E$2:$Q$9,ROWS($E$2:E9),0)</f>
         <v>7584963214</v>
       </c>
-      <c r="F29" s="70"/>
-      <c r="G29" s="70"/>
+      <c r="F29" s="65"/>
+      <c r="G29" s="65"/>
     </row>
     <row r="30" spans="3:7" ht="14.25" customHeight="1"/>
     <row r="31" spans="3:7" ht="14.25" customHeight="1"/>
     <row r="32" spans="3:7" ht="14.25" customHeight="1"/>
     <row r="33" spans="2:9" ht="14.25" customHeight="1" thickBot="1"/>
     <row r="34" spans="2:9" ht="68.25" customHeight="1">
-      <c r="B34" s="126" t="s">
-        <v>97</v>
-      </c>
-      <c r="C34" s="127"/>
-      <c r="D34" s="127"/>
-      <c r="E34" s="127"/>
-      <c r="F34" s="127"/>
-      <c r="G34" s="127"/>
-      <c r="H34" s="127"/>
-      <c r="I34" s="54" t="str">
+      <c r="B34" s="122" t="s">
+        <v>80</v>
+      </c>
+      <c r="C34" s="123"/>
+      <c r="D34" s="123"/>
+      <c r="E34" s="123"/>
+      <c r="F34" s="123"/>
+      <c r="G34" s="123"/>
+      <c r="H34" s="123"/>
+      <c r="I34" s="53" t="str">
         <f t="shared" ref="I34:I40" si="0">HLOOKUP($D$12,$E$2:$Q$9,ROW(E2),0)</f>
         <v>Kapil Singh</v>
       </c>
     </row>
     <row r="35" spans="2:9">
-      <c r="B35" s="56"/>
-      <c r="I35" s="55">
+      <c r="B35" s="55"/>
+      <c r="I35" s="54">
         <f t="shared" si="0"/>
         <v>28</v>
       </c>
     </row>
     <row r="36" spans="2:9">
-      <c r="B36" s="56"/>
-      <c r="I36" s="55" t="str">
+      <c r="B36" s="55"/>
+      <c r="I36" s="54" t="str">
         <f t="shared" si="0"/>
         <v>CAD Designer</v>
       </c>
     </row>
     <row r="37" spans="2:9">
-      <c r="B37" s="56"/>
-      <c r="I37" s="55" t="str">
+      <c r="B37" s="55"/>
+      <c r="I37" s="54" t="str">
         <f t="shared" si="0"/>
         <v>Technical</v>
       </c>
     </row>
     <row r="38" spans="2:9">
-      <c r="B38" s="56"/>
-      <c r="I38" s="55">
+      <c r="B38" s="55"/>
+      <c r="I38" s="54">
         <f t="shared" si="0"/>
         <v>20000</v>
       </c>
     </row>
     <row r="39" spans="2:9">
-      <c r="B39" s="56"/>
-      <c r="I39" s="55" t="str">
+      <c r="B39" s="55"/>
+      <c r="I39" s="54" t="str">
         <f t="shared" si="0"/>
         <v>Indore</v>
       </c>
     </row>
     <row r="40" spans="2:9" ht="15" thickBot="1">
-      <c r="B40" s="57"/>
-      <c r="C40" s="58"/>
-      <c r="D40" s="58"/>
-      <c r="E40" s="58"/>
-      <c r="F40" s="58"/>
-      <c r="G40" s="58"/>
-      <c r="H40" s="58"/>
-      <c r="I40" s="60">
+      <c r="B40" s="56"/>
+      <c r="C40" s="57"/>
+      <c r="D40" s="57"/>
+      <c r="E40" s="57"/>
+      <c r="F40" s="57"/>
+      <c r="G40" s="57"/>
+      <c r="H40" s="57"/>
+      <c r="I40" s="59">
         <f t="shared" si="0"/>
         <v>7584963214</v>
       </c>
@@ -6144,7 +5928,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet8.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0700-000000000000}">
   <dimension ref="A1:S21"/>
   <sheetFormatPr defaultColWidth="8.6328125" defaultRowHeight="14.5"/>
@@ -6172,26 +5956,26 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:19" ht="14.25" customHeight="1">
-      <c r="A1" s="139" t="s">
+      <c r="A1" s="121" t="s">
         <v>0</v>
       </c>
-      <c r="B1" s="139"/>
-      <c r="C1" s="139"/>
-      <c r="D1" s="139"/>
-      <c r="E1" s="139"/>
-      <c r="F1" s="139"/>
-      <c r="G1" s="139"/>
-      <c r="H1" s="139"/>
+      <c r="B1" s="121"/>
+      <c r="C1" s="121"/>
+      <c r="D1" s="121"/>
+      <c r="E1" s="121"/>
+      <c r="F1" s="121"/>
+      <c r="G1" s="121"/>
+      <c r="H1" s="121"/>
     </row>
     <row r="2" spans="1:19" ht="14.25" customHeight="1">
-      <c r="A2" s="139"/>
-      <c r="B2" s="139"/>
-      <c r="C2" s="139"/>
-      <c r="D2" s="139"/>
-      <c r="E2" s="139"/>
-      <c r="F2" s="139"/>
-      <c r="G2" s="139"/>
-      <c r="H2" s="139"/>
+      <c r="A2" s="121"/>
+      <c r="B2" s="121"/>
+      <c r="C2" s="121"/>
+      <c r="D2" s="121"/>
+      <c r="E2" s="121"/>
+      <c r="F2" s="121"/>
+      <c r="G2" s="121"/>
+      <c r="H2" s="121"/>
     </row>
     <row r="3" spans="1:19" ht="23.25" customHeight="1" thickBot="1">
       <c r="A3" s="1" t="s">
@@ -6218,14 +6002,14 @@
       <c r="H3" s="1" t="s">
         <v>8</v>
       </c>
-      <c r="L3" s="83"/>
-      <c r="M3" s="83"/>
-      <c r="N3" s="83"/>
-      <c r="O3" s="83"/>
-      <c r="P3" s="83"/>
-      <c r="Q3" s="83"/>
-      <c r="R3" s="83"/>
-      <c r="S3" s="83"/>
+      <c r="L3" s="78"/>
+      <c r="M3" s="78"/>
+      <c r="N3" s="78"/>
+      <c r="O3" s="78"/>
+      <c r="P3" s="78"/>
+      <c r="Q3" s="78"/>
+      <c r="R3" s="78"/>
+      <c r="S3" s="78"/>
     </row>
     <row r="4" spans="1:19" ht="21" customHeight="1">
       <c r="A4" s="3">
@@ -6252,16 +6036,16 @@
       <c r="H4" s="5">
         <v>8877456987</v>
       </c>
-      <c r="L4" s="87" t="s">
-        <v>98</v>
-      </c>
-      <c r="M4" s="88"/>
-      <c r="N4" s="88"/>
-      <c r="O4" s="88"/>
-      <c r="P4" s="88"/>
-      <c r="Q4" s="88"/>
-      <c r="R4" s="88"/>
-      <c r="S4" s="89"/>
+      <c r="L4" s="82" t="s">
+        <v>81</v>
+      </c>
+      <c r="M4" s="83"/>
+      <c r="N4" s="83"/>
+      <c r="O4" s="83"/>
+      <c r="P4" s="83"/>
+      <c r="Q4" s="83"/>
+      <c r="R4" s="83"/>
+      <c r="S4" s="84"/>
     </row>
     <row r="5" spans="1:19" ht="21" customHeight="1">
       <c r="A5" s="3">
@@ -6288,8 +6072,8 @@
       <c r="H5" s="5">
         <v>8569741235</v>
       </c>
-      <c r="L5" s="61" t="s">
-        <v>92</v>
+      <c r="L5" s="60" t="s">
+        <v>75</v>
       </c>
       <c r="M5" s="3"/>
       <c r="N5" s="3"/>
@@ -6297,7 +6081,7 @@
       <c r="P5" s="3"/>
       <c r="Q5" s="3"/>
       <c r="R5" s="3"/>
-      <c r="S5" s="90"/>
+      <c r="S5" s="85"/>
     </row>
     <row r="6" spans="1:19" ht="21" customHeight="1" thickBot="1">
       <c r="A6" s="3">
@@ -6324,34 +6108,34 @@
       <c r="H6" s="5">
         <v>7584963214</v>
       </c>
-      <c r="L6" s="91">
+      <c r="L6" s="86">
         <v>20015</v>
       </c>
-      <c r="M6" s="92" t="str">
+      <c r="M6" s="87" t="str">
         <f>VLOOKUP(L6,A3:H15,2,0)</f>
         <v>Ali Asgar</v>
       </c>
-      <c r="N6" s="92">
+      <c r="N6" s="87">
         <f>VLOOKUP(L6,A3:H15,3,0)</f>
         <v>27</v>
       </c>
-      <c r="O6" s="92" t="str">
+      <c r="O6" s="87" t="str">
         <f>VLOOKUP(L6,A3:H15,4,0)</f>
         <v>Accountant</v>
       </c>
-      <c r="P6" s="92" t="str">
+      <c r="P6" s="87" t="str">
         <f>VLOOKUP(L6,A3:H15,5,0)</f>
         <v>Finance</v>
       </c>
-      <c r="Q6" s="92">
+      <c r="Q6" s="87">
         <f>VLOOKUP(L6,A3:H15,6,0)</f>
         <v>15000</v>
       </c>
-      <c r="R6" s="92" t="str">
+      <c r="R6" s="87" t="str">
         <f>VLOOKUP(L6,A3:H15,7,0)</f>
         <v>Bhopal</v>
       </c>
-      <c r="S6" s="93">
+      <c r="S6" s="88">
         <f>VLOOKUP(L6,A3:H15,8,0)</f>
         <v>7788994455</v>
       </c>
@@ -6382,19 +6166,19 @@
         <v>7788994455</v>
       </c>
       <c r="J7" s="2"/>
-      <c r="L7" s="94" t="s">
-        <v>99</v>
-      </c>
-      <c r="M7" s="82">
+      <c r="L7" s="89" t="s">
+        <v>82</v>
+      </c>
+      <c r="M7" s="77">
         <f>VLOOKUP(B8,B3:H15,5,0)</f>
         <v>20000</v>
       </c>
-      <c r="N7" s="98"/>
-      <c r="O7" s="98"/>
-      <c r="P7" s="98"/>
-      <c r="Q7" s="98"/>
-      <c r="R7" s="99"/>
-      <c r="S7" s="100"/>
+      <c r="N7" s="93"/>
+      <c r="O7" s="93"/>
+      <c r="P7" s="93"/>
+      <c r="Q7" s="93"/>
+      <c r="R7" s="94"/>
+      <c r="S7" s="95"/>
     </row>
     <row r="8" spans="1:19" ht="21" customHeight="1" thickBot="1">
       <c r="A8" s="3">
@@ -6447,16 +6231,16 @@
       <c r="H9" s="5">
         <v>9874563214</v>
       </c>
-      <c r="L9" s="84" t="s">
-        <v>106</v>
-      </c>
-      <c r="M9" s="85"/>
-      <c r="N9" s="85"/>
-      <c r="O9" s="85"/>
-      <c r="P9" s="85"/>
-      <c r="Q9" s="85"/>
-      <c r="R9" s="85"/>
-      <c r="S9" s="86"/>
+      <c r="L9" s="79" t="s">
+        <v>89</v>
+      </c>
+      <c r="M9" s="80"/>
+      <c r="N9" s="80"/>
+      <c r="O9" s="80"/>
+      <c r="P9" s="80"/>
+      <c r="Q9" s="80"/>
+      <c r="R9" s="80"/>
+      <c r="S9" s="81"/>
     </row>
     <row r="10" spans="1:19" ht="21" customHeight="1">
       <c r="A10" s="3">
@@ -6483,7 +6267,7 @@
       <c r="H10" s="5">
         <v>8974563214</v>
       </c>
-      <c r="L10" s="56">
+      <c r="L10" s="55">
         <v>20016</v>
       </c>
       <c r="M10" s="3" t="str">
@@ -6501,7 +6285,7 @@
       </c>
       <c r="Q10" s="3"/>
       <c r="R10" s="3"/>
-      <c r="S10" s="90"/>
+      <c r="S10" s="85"/>
     </row>
     <row r="11" spans="1:19" ht="21" customHeight="1">
       <c r="A11" s="3">
@@ -6528,7 +6312,7 @@
       <c r="H11" s="5">
         <v>8745968745</v>
       </c>
-      <c r="L11" s="56">
+      <c r="L11" s="55">
         <v>20017</v>
       </c>
       <c r="M11" s="3" t="str">
@@ -6544,7 +6328,7 @@
       <c r="P11" s="5">
         <v>9874563214</v>
       </c>
-      <c r="S11" s="55"/>
+      <c r="S11" s="54"/>
     </row>
     <row r="12" spans="1:19" ht="21" customHeight="1" thickBot="1">
       <c r="A12" s="3">
@@ -6571,25 +6355,25 @@
       <c r="H12" s="5">
         <v>9874569874</v>
       </c>
-      <c r="L12" s="57">
+      <c r="L12" s="56">
         <v>20020</v>
       </c>
-      <c r="M12" s="92" t="str">
+      <c r="M12" s="87" t="str">
         <f t="array" ref="M12:P12">VLOOKUP(A10,A5:H17,{2,4,6,8},0)</f>
         <v>Ravi Verma</v>
       </c>
-      <c r="N12" s="92" t="str">
+      <c r="N12" s="87" t="str">
         <v>CAD Designer</v>
       </c>
-      <c r="O12" s="92">
+      <c r="O12" s="87">
         <v>21000</v>
       </c>
-      <c r="P12" s="95">
+      <c r="P12" s="90">
         <v>8974563214</v>
       </c>
-      <c r="Q12" s="92"/>
-      <c r="R12" s="92"/>
-      <c r="S12" s="96"/>
+      <c r="Q12" s="87"/>
+      <c r="R12" s="87"/>
+      <c r="S12" s="91"/>
     </row>
     <row r="13" spans="1:19" ht="21" customHeight="1" thickBot="1">
       <c r="A13" s="3">
@@ -6616,13 +6400,13 @@
       <c r="H13" s="5">
         <v>8574965874</v>
       </c>
-      <c r="M13" s="101"/>
-      <c r="N13" s="101"/>
-      <c r="O13" s="101"/>
-      <c r="P13" s="101"/>
-      <c r="Q13" s="101"/>
-      <c r="R13" s="101"/>
-      <c r="S13" s="97"/>
+      <c r="M13" s="96"/>
+      <c r="N13" s="96"/>
+      <c r="O13" s="96"/>
+      <c r="P13" s="96"/>
+      <c r="Q13" s="96"/>
+      <c r="R13" s="96"/>
+      <c r="S13" s="92"/>
     </row>
     <row r="14" spans="1:19" ht="21" customHeight="1" thickBot="1">
       <c r="A14" s="3">
@@ -6649,26 +6433,26 @@
       <c r="H14" s="5">
         <v>8521479632</v>
       </c>
-      <c r="L14" s="73" t="s">
-        <v>100</v>
-      </c>
-      <c r="M14" s="72">
+      <c r="L14" s="68" t="s">
+        <v>83</v>
+      </c>
+      <c r="M14" s="67">
         <f t="array" ref="M14:R14">VLOOKUP(B12,B3:H15,{2,3,4,5,6,7},0)</f>
         <v>28</v>
       </c>
-      <c r="N14" s="72" t="str">
+      <c r="N14" s="67" t="str">
         <v>Accountant</v>
       </c>
-      <c r="O14" s="72" t="str">
+      <c r="O14" s="67" t="str">
         <v>Finance</v>
       </c>
-      <c r="P14" s="72">
+      <c r="P14" s="67">
         <v>40500</v>
       </c>
-      <c r="Q14" s="72" t="str">
+      <c r="Q14" s="67" t="str">
         <v>Indore</v>
       </c>
-      <c r="R14" s="102">
+      <c r="R14" s="97">
         <v>9874569874</v>
       </c>
     </row>
@@ -6700,53 +6484,53 @@
       <c r="S15" s="3"/>
     </row>
     <row r="16" spans="1:19">
-      <c r="L16" s="74" t="s">
-        <v>101</v>
-      </c>
-      <c r="M16" s="78"/>
-      <c r="N16" s="78"/>
-      <c r="O16" s="79"/>
-      <c r="P16" s="79"/>
-      <c r="Q16" s="79"/>
-      <c r="R16" s="79"/>
-      <c r="S16" s="54"/>
+      <c r="L16" s="69" t="s">
+        <v>84</v>
+      </c>
+      <c r="M16" s="73"/>
+      <c r="N16" s="73"/>
+      <c r="O16" s="74"/>
+      <c r="P16" s="74"/>
+      <c r="Q16" s="74"/>
+      <c r="R16" s="74"/>
+      <c r="S16" s="53"/>
     </row>
     <row r="17" spans="12:19" ht="27.75" customHeight="1">
-      <c r="L17" s="56"/>
-      <c r="M17" s="80" t="s">
-        <v>92</v>
-      </c>
-      <c r="N17" s="81" t="s">
+      <c r="L17" s="55"/>
+      <c r="M17" s="75" t="s">
+        <v>75</v>
+      </c>
+      <c r="N17" s="76" t="s">
         <v>2</v>
       </c>
-      <c r="S17" s="55"/>
+      <c r="S17" s="54"/>
     </row>
     <row r="18" spans="12:19" ht="36" customHeight="1" thickBot="1">
-      <c r="L18" s="57"/>
-      <c r="M18" s="58">
+      <c r="L18" s="56"/>
+      <c r="M18" s="57">
         <v>20017</v>
       </c>
-      <c r="N18" s="58" t="str">
+      <c r="N18" s="57" t="str">
         <f>VLOOKUP(M18,A3:H15,MATCH(N17,A3:H3,0),0)</f>
         <v>Mohan Patel</v>
       </c>
-      <c r="O18" s="58"/>
-      <c r="P18" s="58"/>
-      <c r="Q18" s="58"/>
-      <c r="R18" s="58"/>
-      <c r="S18" s="60"/>
+      <c r="O18" s="57"/>
+      <c r="P18" s="57"/>
+      <c r="Q18" s="57"/>
+      <c r="R18" s="57"/>
+      <c r="S18" s="59"/>
     </row>
     <row r="19" spans="12:19" ht="14.25" customHeight="1"/>
     <row r="20" spans="12:19" ht="14.25" customHeight="1" thickBot="1"/>
     <row r="21" spans="12:19" ht="36" customHeight="1" thickBot="1">
-      <c r="L21" s="104" t="s">
-        <v>102</v>
-      </c>
-      <c r="M21" s="72">
+      <c r="L21" s="99" t="s">
+        <v>85</v>
+      </c>
+      <c r="M21" s="67">
         <f>MATCH(B3,A3:H3,0)</f>
         <v>2</v>
       </c>
-      <c r="N21" s="103"/>
+      <c r="N21" s="98"/>
       <c r="O21" s="2"/>
       <c r="P21" s="2"/>
     </row>

</xml_diff>